<commit_message>
Checkpoint: PreA sheet built with grouped holders and cross-sheet refs
</commit_message>
<xml_diff>
--- a/runs/20260414-110202/models/model.xlsx
+++ b/runs/20260414-110202/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E63652D-FA7F-0246-BEEB-028D122B5548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73FD80AC-9303-764F-8D0C-9F1FD0AADCE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="119" r:id="rId1"/>
     <sheet name="Detailed Cap Table" sheetId="120" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="122" r:id="rId3"/>
+    <sheet name="PreA" sheetId="123" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>Total</t>
   </si>
@@ -193,17 +194,84 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>SAFE Post-Money Valuation Cap</t>
+  </si>
+  <si>
+    <t>Common</t>
+  </si>
+  <si>
+    <t>Other Common Shareholders</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Other SAFE Investors</t>
+  </si>
+  <si>
+    <t>Invested</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
+    <t>THINK MORE SECURITY &amp; 1011 VENTURES PRE-SERIES A</t>
+  </si>
+  <si>
+    <t>PRE-SERIES A CAPITALIZATION</t>
+  </si>
+  <si>
+    <t>ESOP Outstanding</t>
+  </si>
+  <si>
+    <t>SAFE Investors:</t>
+  </si>
+  <si>
+    <t>Implied Price per Share</t>
+  </si>
+  <si>
+    <t>Company Capitalization (pre-A)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +407,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -352,6 +445,13 @@
       <family val="1"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -539,7 +639,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -654,6 +754,147 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -699,30 +940,125 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1144,518 +1480,518 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="A1" s="12"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="2" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1" t="s">
+      <c r="A4" s="12"/>
+      <c r="B4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="14">
         <v>3600000</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3">
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="15">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1" t="s">
+      <c r="A5" s="12"/>
+      <c r="B5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="14">
         <v>3600000</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3">
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="15">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
+      <c r="A6" s="12"/>
+      <c r="B6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="14">
         <v>222187</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3">
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="15">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="14">
         <v>592500</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3">
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="15">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
+      <c r="A8" s="12"/>
+      <c r="B8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="14">
         <v>592500</v>
       </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3">
+      <c r="D8" s="14"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="15">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1" t="s">
+      <c r="A9" s="12"/>
+      <c r="B9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="14">
         <v>13500</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="14">
         <v>98900</v>
       </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3">
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="15">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1" t="s">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="14">
         <v>9000</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3">
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="15">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1" t="s">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3">
+      <c r="C11" s="14"/>
+      <c r="D11" s="14">
         <v>95000</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3">
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="15">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1" t="s">
+      <c r="A12" s="12"/>
+      <c r="B12" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3">
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14">
         <v>25000</v>
       </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3">
+      <c r="F12" s="14"/>
+      <c r="G12" s="14">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="15">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3">
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14">
         <v>41562</v>
       </c>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3">
+      <c r="F13" s="14"/>
+      <c r="G13" s="14">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="15">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1" t="s">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3">
+      <c r="C14" s="14"/>
+      <c r="D14" s="14">
         <v>285000</v>
       </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3">
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="14">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="15">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1" t="s">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3">
+      <c r="C15" s="14"/>
+      <c r="D15" s="14">
         <v>50000</v>
       </c>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3">
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="15">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3">
+      <c r="C16" s="14"/>
+      <c r="D16" s="14">
         <v>285000</v>
       </c>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3">
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="15">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1" t="s">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3">
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14">
         <v>96186</v>
       </c>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3">
+      <c r="F17" s="14"/>
+      <c r="G17" s="14">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="15">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1" t="s">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3">
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14">
         <v>48095</v>
       </c>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3">
+      <c r="F18" s="14"/>
+      <c r="G18" s="14">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="15">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1" t="s">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3">
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14">
         <v>12395</v>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" s="14">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="15">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1" t="s">
+      <c r="A20" s="12"/>
+      <c r="B20" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3">
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14">
         <v>8333</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="14">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="15">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1" t="s">
+      <c r="A21" s="12"/>
+      <c r="B21" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3">
+      <c r="C21" s="14"/>
+      <c r="D21" s="14">
         <v>65105</v>
       </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3">
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="15">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="2" t="s">
+      <c r="A23" s="12"/>
+      <c r="B23" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="36">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="36">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="8">
+      <c r="E23" s="36">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="36">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="8">
+      <c r="G23" s="36">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1676,476 +2012,906 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="6"/>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
+      <c r="A1" s="18"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="18"/>
+      <c r="B3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="6"/>
-      <c r="E3" s="2" t="s">
+      <c r="D3" s="18"/>
+      <c r="E3" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="1" t="s">
+      <c r="A4" s="18"/>
+      <c r="B4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="17">
         <v>25000</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="1" t="s">
+      <c r="A5" s="18"/>
+      <c r="B5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="17">
         <v>25000</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="1" t="s">
+      <c r="A6" s="18"/>
+      <c r="B6" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="17">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="1" t="s">
+      <c r="A7" s="18"/>
+      <c r="B7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="17">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
-      <c r="B8" s="1" t="s">
+      <c r="A8" s="18"/>
+      <c r="B8" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="17">
         <v>16566</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="6"/>
-      <c r="B9" s="1" t="s">
+      <c r="A9" s="18"/>
+      <c r="B9" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="17">
         <v>250000</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="6"/>
-      <c r="B10" s="1" t="s">
+      <c r="A10" s="18"/>
+      <c r="B10" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="17">
         <v>100000</v>
       </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="6"/>
-      <c r="B11" s="1" t="s">
+      <c r="A11" s="18"/>
+      <c r="B11" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="17">
         <v>300000</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1" t="s">
+      <c r="D11" s="12"/>
+      <c r="E11" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="6"/>
-      <c r="B12" s="1" t="s">
+      <c r="A12" s="18"/>
+      <c r="B12" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="17">
         <v>37500</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1" t="s">
+      <c r="D12" s="12"/>
+      <c r="E12" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="18"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="6"/>
-      <c r="B13" s="1" t="s">
+      <c r="A13" s="18"/>
+      <c r="B13" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="17">
         <v>250000</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="6"/>
-      <c r="B14" s="1" t="s">
+      <c r="A14" s="18"/>
+      <c r="B14" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="17">
         <v>100000</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="6"/>
-      <c r="B15" s="1" t="s">
+      <c r="A15" s="18"/>
+      <c r="B15" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="17">
         <v>41164</v>
       </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="6"/>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="18"/>
+      <c r="B16" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="17">
         <v>2328778</v>
       </c>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="B17" s="1" t="s">
+      <c r="A17" s="18"/>
+      <c r="B17" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="17">
         <v>1506000</v>
       </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1" t="s">
+      <c r="D17" s="12"/>
+      <c r="E17" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="6"/>
-      <c r="B18" s="1" t="s">
+      <c r="A18" s="18"/>
+      <c r="B18" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="17">
         <v>50000</v>
       </c>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="6"/>
-      <c r="B19" s="1" t="s">
+      <c r="A19" s="18"/>
+      <c r="B19" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="17">
         <v>212500</v>
       </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="12"/>
+      <c r="E19" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
+      <c r="K19" s="18"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="6"/>
-      <c r="B20" s="1" t="s">
+      <c r="A20" s="18"/>
+      <c r="B20" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="17">
         <v>25000</v>
       </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="6"/>
-      <c r="B21" s="1" t="s">
+      <c r="A21" s="18"/>
+      <c r="B21" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="17">
         <v>61746</v>
       </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="18"/>
+      <c r="K21" s="18"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="6"/>
-      <c r="B22" s="1" t="s">
+      <c r="A22" s="18"/>
+      <c r="B22" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="17">
         <v>100000</v>
       </c>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
-      <c r="B23" s="1" t="s">
+      <c r="A23" s="18"/>
+      <c r="B23" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="17">
         <v>100000</v>
       </c>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="B24" s="1" t="s">
+      <c r="A24" s="18"/>
+      <c r="B24" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="17">
         <v>61746</v>
       </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="6"/>
-      <c r="B25" s="1" t="s">
+      <c r="A25" s="18"/>
+      <c r="B25" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="17">
         <v>250000</v>
       </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1" t="s">
+      <c r="D25" s="12"/>
+      <c r="E25" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="6"/>
-      <c r="B27" s="1" t="s">
+      <c r="A27" s="18"/>
+      <c r="B27" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="17">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B125570-B131-A546-AB8D-19A0B295BDA7}">
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="0.5" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+    </row>
+    <row r="5" spans="1:7" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+    </row>
+    <row r="6" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="31"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="42" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="43" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="30"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="3">
+        <f>'Detailed Cap Table'!C4</f>
+        <v>3600000</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="5">
+        <f>C10</f>
+        <v>3600000</v>
+      </c>
+      <c r="G10" s="33">
+        <f>F10/$F$21</f>
+        <v>0.36959987630724139</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3">
+        <f>'Detailed Cap Table'!C5</f>
+        <v>3600000</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="5">
+        <f>C11</f>
+        <v>3600000</v>
+      </c>
+      <c r="G11" s="33">
+        <f>F11/$F$21</f>
+        <v>0.36959987630724139</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="3">
+        <f>'Detailed Cap Table'!C6+'Detailed Cap Table'!C7+'Detailed Cap Table'!C8+'Detailed Cap Table'!C9+'Detailed Cap Table'!C10+'Detailed Cap Table'!F19+'Detailed Cap Table'!F20</f>
+        <v>1450415</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="5">
+        <f>C12</f>
+        <v>1450415</v>
+      </c>
+      <c r="G12" s="33">
+        <f>F12/$F$21</f>
+        <v>0.14890922349837987</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="3">
+        <f>SUM('Detailed Cap Table'!D4:D20)+SUM('Detailed Cap Table'!E4:E20)</f>
+        <v>1024743</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="5">
+        <f>C13</f>
+        <v>1024743</v>
+      </c>
+      <c r="G13" s="33">
+        <f>F13/$F$21</f>
+        <v>0.10520691279075318</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="38">
+        <f>'Detailed Cap Table'!D21</f>
+        <v>65105</v>
+      </c>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="39">
+        <f>C14</f>
+        <v>65105</v>
+      </c>
+      <c r="G14" s="40">
+        <f>F14/$F$21</f>
+        <v>6.6841110963841528E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="6">
+        <f>SUM(C10:C14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="6">
+        <f>SUM(F10:F14)</f>
+        <v>9740263</v>
+      </c>
+      <c r="G15" s="34">
+        <f>SUM(G10:G14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="33"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="7">
+        <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
+        <v>8000000</v>
+      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="5">
+        <v>0</v>
+      </c>
+      <c r="G17" s="33">
+        <f>F17/$F$21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="7">
+        <f>'SAFE Investments'!C27-D17</f>
+        <v>1825000</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+      <c r="G18" s="33">
+        <f>F18/$F$21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="33"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="33"/>
+    </row>
+    <row r="21" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="9">
+        <f>C15</f>
+        <v>9740263</v>
+      </c>
+      <c r="D21" s="10">
+        <f>SUM(D17:D18)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E21" s="11"/>
+      <c r="F21" s="9">
+        <f>F15</f>
+        <v>9740263</v>
+      </c>
+      <c r="G21" s="41">
+        <f>SUM(G10:G14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="4"/>
+      <c r="D24" s="16">
+        <v>50000000</v>
+      </c>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+    </row>
+    <row r="25" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="5">
+        <f>F21</f>
+        <v>9740263</v>
+      </c>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Series A sheet - fixed totals double-counting
</commit_message>
<xml_diff>
--- a/runs/20260414-110202/models/model.xlsx
+++ b/runs/20260414-110202/models/model.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73FD80AC-9303-764F-8D0C-9F1FD0AADCE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5988BF2C-0D55-9F4E-B96A-D7ECCC229F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="119" r:id="rId1"/>
     <sheet name="Detailed Cap Table" sheetId="120" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="122" r:id="rId3"/>
     <sheet name="PreA" sheetId="123" r:id="rId4"/>
+    <sheet name="Series A" sheetId="124" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="96">
   <si>
     <t>Total</t>
   </si>
@@ -194,6 +195,9 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t>Series A</t>
+  </si>
+  <si>
     <t>Total Capitalization</t>
   </si>
   <si>
@@ -203,6 +207,12 @@
     <t>$</t>
   </si>
   <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
     <t>Total FD</t>
   </si>
   <si>
@@ -212,6 +222,12 @@
     <t>Shares</t>
   </si>
   <si>
+    <t>SAFE Shares</t>
+  </si>
+  <si>
+    <t>Pre A</t>
+  </si>
+  <si>
     <t>FD</t>
   </si>
   <si>
@@ -221,15 +237,48 @@
     <t>Total Common</t>
   </si>
   <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>1011 Ventures</t>
+  </si>
+  <si>
+    <t>Other Series A Investors</t>
+  </si>
+  <si>
     <t>Totals</t>
   </si>
   <si>
+    <t>Price per Share</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>Total Raised</t>
+  </si>
+  <si>
+    <t>1011 Ventures Investment</t>
+  </si>
+  <si>
     <t>SAFE Post-Money Valuation Cap</t>
   </si>
   <si>
     <t>Common</t>
   </si>
   <si>
+    <t>Option</t>
+  </si>
+  <si>
+    <t>Pre SAFE</t>
+  </si>
+  <si>
     <t>Other Common Shareholders</t>
   </si>
   <si>
@@ -261,17 +310,33 @@
   </si>
   <si>
     <t>Company Capitalization (pre-A)</t>
+  </si>
+  <si>
+    <t>THINK MORE SECURITY</t>
+  </si>
+  <si>
+    <t>1011 VENTURES SERIES A</t>
+  </si>
+  <si>
+    <t>% Ownership Check</t>
+  </si>
+  <si>
+    <t>Option Pool Expansion (% of post-money FD)</t>
+  </si>
+  <si>
+    <t>Accomplice New Money</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0000"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -448,6 +513,13 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Garamond"/>
       <family val="1"/>
     </font>
@@ -639,7 +711,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -784,6 +856,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -885,6 +966,17 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="medium">
         <color rgb="FF000000"/>
@@ -940,12 +1032,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -964,6 +1058,12 @@
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -985,80 +1085,104 @@
     <xf numFmtId="10" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="19" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1480,518 +1604,518 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="12"/>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
+      <c r="A1" s="16"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="13" t="s">
+      <c r="A2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13" t="s">
+      <c r="A3" s="16"/>
+      <c r="B3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="16"/>
+      <c r="B4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="18">
         <v>3600000</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14">
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="19">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
+      <c r="I4" s="16"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12" t="s">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="18">
         <v>3600000</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14">
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="19">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12" t="s">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="18">
         <v>222187</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14">
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="19">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="18">
         <v>592500</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14">
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="19">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="18">
         <v>592500</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14">
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="15">
+      <c r="H8" s="19">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12" t="s">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="18">
         <v>13500</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="18">
         <v>98900</v>
       </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14">
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="15">
+      <c r="H9" s="19">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="18">
         <v>9000</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14">
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="15">
+      <c r="H10" s="19">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14">
+      <c r="C11" s="18"/>
+      <c r="D11" s="18">
         <v>95000</v>
       </c>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14">
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H11" s="19">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12" t="s">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14">
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18">
         <v>25000</v>
       </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14">
+      <c r="F12" s="18"/>
+      <c r="G12" s="18">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="19">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12" t="s">
+      <c r="A13" s="16"/>
+      <c r="B13" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14">
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18">
         <v>41562</v>
       </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14">
+      <c r="F13" s="18"/>
+      <c r="G13" s="18">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="19">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12" t="s">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14">
+      <c r="C14" s="18"/>
+      <c r="D14" s="18">
         <v>285000</v>
       </c>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14">
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="19">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12" t="s">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14">
+      <c r="C15" s="18"/>
+      <c r="D15" s="18">
         <v>50000</v>
       </c>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14">
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="19">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12" t="s">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14">
+      <c r="C16" s="18"/>
+      <c r="D16" s="18">
         <v>285000</v>
       </c>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14">
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="19">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12" t="s">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14">
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18">
         <v>96186</v>
       </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14">
+      <c r="F17" s="18"/>
+      <c r="G17" s="18">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="15">
+      <c r="H17" s="19">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12" t="s">
+      <c r="A18" s="16"/>
+      <c r="B18" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14">
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18">
         <v>48095</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14">
+      <c r="F18" s="18"/>
+      <c r="G18" s="18">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="19">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12" t="s">
+      <c r="A19" s="16"/>
+      <c r="B19" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14">
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18">
         <v>12395</v>
       </c>
-      <c r="G19" s="14">
+      <c r="G19" s="18">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="19">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12" t="s">
+      <c r="A20" s="16"/>
+      <c r="B20" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14">
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18">
         <v>8333</v>
       </c>
-      <c r="G20" s="14">
+      <c r="G20" s="18">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="19">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12" t="s">
+      <c r="A21" s="16"/>
+      <c r="B21" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14">
+      <c r="C21" s="18"/>
+      <c r="D21" s="18">
         <v>65105</v>
       </c>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14">
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H21" s="19">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12"/>
-      <c r="B23" s="13" t="s">
+      <c r="A23" s="16"/>
+      <c r="B23" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="36">
+      <c r="C23" s="46">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="36">
+      <c r="D23" s="46">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="36">
+      <c r="E23" s="46">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="36">
+      <c r="F23" s="46">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="36">
+      <c r="G23" s="46">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2012,476 +2136,476 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="18"/>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
+      <c r="A1" s="24"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
+      <c r="A2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="18"/>
-      <c r="B3" s="13" t="s">
+      <c r="A3" s="24"/>
+      <c r="B3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="18"/>
-      <c r="E3" s="13" t="s">
+      <c r="D3" s="24"/>
+      <c r="E3" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="18"/>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="24"/>
+      <c r="B4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="22">
         <v>25000</v>
       </c>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="18"/>
-      <c r="B5" s="12" t="s">
+      <c r="A5" s="24"/>
+      <c r="B5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="22">
         <v>25000</v>
       </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="18"/>
-      <c r="B6" s="12" t="s">
+      <c r="A6" s="24"/>
+      <c r="B6" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="22">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="18"/>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="24"/>
+      <c r="B7" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="22">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="18"/>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="24"/>
+      <c r="B8" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="22">
         <v>16566</v>
       </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="18"/>
-      <c r="B9" s="12" t="s">
+      <c r="A9" s="24"/>
+      <c r="B9" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="22">
         <v>250000</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="18"/>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="24"/>
+      <c r="B10" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="22">
         <v>100000</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="24"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="18"/>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="24"/>
+      <c r="B11" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="22">
         <v>300000</v>
       </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12" t="s">
+      <c r="D11" s="16"/>
+      <c r="E11" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="18"/>
-      <c r="B12" s="12" t="s">
+      <c r="A12" s="24"/>
+      <c r="B12" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="22">
         <v>37500</v>
       </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12" t="s">
+      <c r="D12" s="16"/>
+      <c r="E12" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="18"/>
-      <c r="B13" s="12" t="s">
+      <c r="A13" s="24"/>
+      <c r="B13" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="22">
         <v>250000</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="18"/>
-      <c r="B14" s="12" t="s">
+      <c r="A14" s="24"/>
+      <c r="B14" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="22">
         <v>100000</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="18"/>
-      <c r="B15" s="12" t="s">
+      <c r="A15" s="24"/>
+      <c r="B15" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="22">
         <v>41164</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="24"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="18"/>
-      <c r="B16" s="12" t="s">
+      <c r="A16" s="24"/>
+      <c r="B16" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="22">
         <v>2328778</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="18"/>
-      <c r="B17" s="12" t="s">
+      <c r="A17" s="24"/>
+      <c r="B17" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="22">
         <v>1506000</v>
       </c>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12" t="s">
+      <c r="D17" s="16"/>
+      <c r="E17" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="24"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="18"/>
-      <c r="B18" s="12" t="s">
+      <c r="A18" s="24"/>
+      <c r="B18" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="22">
         <v>50000</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="18"/>
-      <c r="B19" s="12" t="s">
+      <c r="A19" s="24"/>
+      <c r="B19" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="22">
         <v>212500</v>
       </c>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12" t="s">
+      <c r="D19" s="16"/>
+      <c r="E19" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="24"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="18"/>
-      <c r="B20" s="12" t="s">
+      <c r="A20" s="24"/>
+      <c r="B20" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="22">
         <v>25000</v>
       </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="18"/>
-      <c r="B21" s="12" t="s">
+      <c r="A21" s="24"/>
+      <c r="B21" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="22">
         <v>61746</v>
       </c>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="18"/>
-      <c r="B22" s="12" t="s">
+      <c r="A22" s="24"/>
+      <c r="B22" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="22">
         <v>100000</v>
       </c>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="24"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="18"/>
-      <c r="B23" s="12" t="s">
+      <c r="A23" s="24"/>
+      <c r="B23" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="17">
+      <c r="C23" s="22">
         <v>100000</v>
       </c>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="24"/>
+      <c r="K23" s="24"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="18"/>
-      <c r="B24" s="12" t="s">
+      <c r="A24" s="24"/>
+      <c r="B24" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="17">
+      <c r="C24" s="22">
         <v>61746</v>
       </c>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="18"/>
-      <c r="B25" s="12" t="s">
+      <c r="A25" s="24"/>
+      <c r="B25" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="17">
+      <c r="C25" s="22">
         <v>250000</v>
       </c>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12" t="s">
+      <c r="D25" s="16"/>
+      <c r="E25" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="18"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="32"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="18"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="18"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="18"/>
-      <c r="B27" s="12" t="s">
+      <c r="A27" s="24"/>
+      <c r="B27" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="17">
+      <c r="C27" s="22">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="18"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="18"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="K27" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2531,292 +2655,294 @@
     </row>
     <row r="4" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
+      <c r="B4" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
+      <c r="B5" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
     </row>
     <row r="6" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="D6" s="24" t="s">
+      <c r="C6" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" s="31"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="39"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C7" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="29" t="s">
+      <c r="D7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="42" t="s">
-        <v>56</v>
+      <c r="E7" s="6"/>
+      <c r="F7" s="36" t="s">
+        <v>58</v>
+      </c>
+      <c r="G7" s="53" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" s="43" t="s">
-        <v>58</v>
+      <c r="C8" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="54" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="37" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="30"/>
+      <c r="B9" s="47" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="38"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="20" t="s">
+      <c r="B10" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="5">
         <f>'Detailed Cap Table'!C4</f>
         <v>3600000</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="5">
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="7">
         <f>C10</f>
         <v>3600000</v>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="43">
         <f>F10/$F$21</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="5">
         <f>'Detailed Cap Table'!C5</f>
         <v>3600000</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="5">
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7">
         <f>C11</f>
         <v>3600000</v>
       </c>
-      <c r="G11" s="33">
+      <c r="G11" s="43">
         <f>F11/$F$21</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" s="3">
+      <c r="B12" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" s="5">
         <f>'Detailed Cap Table'!C6+'Detailed Cap Table'!C7+'Detailed Cap Table'!C8+'Detailed Cap Table'!C9+'Detailed Cap Table'!C10+'Detailed Cap Table'!F19+'Detailed Cap Table'!F20</f>
         <v>1450415</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="5">
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="7">
         <f>C12</f>
         <v>1450415</v>
       </c>
-      <c r="G12" s="33">
+      <c r="G12" s="43">
         <f>F12/$F$21</f>
         <v>0.14890922349837987</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" s="3">
+      <c r="B13" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="5">
         <f>SUM('Detailed Cap Table'!D4:D20)+SUM('Detailed Cap Table'!E4:E20)</f>
         <v>1024743</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="5">
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="7">
         <f>C13</f>
         <v>1024743</v>
       </c>
-      <c r="G13" s="33">
+      <c r="G13" s="43">
         <f>F13/$F$21</f>
         <v>0.10520691279075318</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="38">
+      <c r="B14" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" s="49">
         <f>'Detailed Cap Table'!D21</f>
         <v>65105</v>
       </c>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="39">
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="50">
         <f>C14</f>
         <v>65105</v>
       </c>
-      <c r="G14" s="40">
+      <c r="G14" s="51">
         <f>F14/$F$21</f>
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="6">
+      <c r="B15" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="8">
         <f>SUM(C10:C14)</f>
         <v>9740263</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="6">
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="8">
         <f>SUM(F10:F14)</f>
         <v>9740263</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="44">
         <f>SUM(G10:G14)</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="33"/>
+      <c r="B16" s="27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="43"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="7">
+      <c r="C17" s="7"/>
+      <c r="D17" s="9">
         <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
         <v>8000000</v>
       </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5">
+      <c r="E17" s="6"/>
+      <c r="F17" s="7">
+        <f>C17</f>
         <v>0</v>
       </c>
-      <c r="G17" s="33">
+      <c r="G17" s="43">
         <f>F17/$F$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="7">
+      <c r="B18" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="9">
         <f>'SAFE Investments'!C27-D17</f>
         <v>1825000</v>
       </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="5">
+      <c r="E18" s="6"/>
+      <c r="F18" s="7">
+        <f>C18</f>
         <v>0</v>
       </c>
-      <c r="G18" s="33">
+      <c r="G18" s="43">
         <f>F18/$F$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="33"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="43"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="33"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="43"/>
     </row>
     <row r="21" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="35" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="9">
+      <c r="B21" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="13">
         <f>C15</f>
         <v>9740263</v>
       </c>
-      <c r="D21" s="10">
+      <c r="D21" s="14">
         <f>SUM(D17:D18)</f>
         <v>9825000</v>
       </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="9">
+      <c r="E21" s="15"/>
+      <c r="F21" s="13">
         <f>F15</f>
         <v>9740263</v>
       </c>
-      <c r="G21" s="41">
+      <c r="G21" s="52">
         <f>SUM(G10:G14)</f>
         <v>1</v>
       </c>
@@ -2824,49 +2950,52 @@
     <row r="22" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
     </row>
     <row r="23" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
+        <v>89</v>
+      </c>
+      <c r="C23" s="11">
+        <f>D24/C25</f>
+        <v>5.1333316153783528</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C24" s="4"/>
-      <c r="D24" s="16">
+        <v>76</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="21">
         <v>50000000</v>
       </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C25" s="5">
+        <v>90</v>
+      </c>
+      <c r="C25" s="7">
         <f>F21</f>
         <v>9740263</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
@@ -2916,4 +3045,916 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DCBE17-48C8-184C-81EE-49F5A5033C50}">
+  <dimension ref="A1:O35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="15.5" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
+    <col min="15" max="15" width="9.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="39"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" s="39"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="M4" s="6"/>
+      <c r="N4" s="29" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4" s="39"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="39" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="6"/>
+      <c r="L5" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="M5" s="6"/>
+      <c r="N5" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="39" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="53" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="J6" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="K6" s="6"/>
+      <c r="L6" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="6"/>
+      <c r="N6" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" s="53" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="47" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
+      <c r="N7" s="33"/>
+      <c r="O7" s="48"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="5">
+        <f>PreA!C10</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="7">
+        <f>C8+E8+G8+J8+L8</f>
+        <v>3600000</v>
+      </c>
+      <c r="O8" s="43">
+        <f ca="1">N8/$N$21</f>
+        <v>0.19407533292814716</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="5">
+        <f>PreA!C11</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="7">
+        <f>C9+E9+G9+J9+L9</f>
+        <v>3600000</v>
+      </c>
+      <c r="O9" s="43">
+        <f ca="1">N9/$N$21</f>
+        <v>0.19407533292814716</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="5">
+        <f>PreA!C12</f>
+        <v>1450415</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="7">
+        <f>C10+E10+G10+J10+L10</f>
+        <v>1450415</v>
+      </c>
+      <c r="O10" s="43">
+        <f ca="1">N10/$N$21</f>
+        <v>7.8191603891382938E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="5">
+        <f>PreA!C13</f>
+        <v>1024743</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="7">
+        <f>C11+E11+G11+J11+L11</f>
+        <v>1024743</v>
+      </c>
+      <c r="O11" s="43">
+        <f ca="1">N11/$N$21</f>
+        <v>5.5243705247441197E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="5">
+        <f>PreA!C14</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="7">
+        <f ca="1">ROUND((C31*(C13+E21+J21)-C12)/(1-C31),0)</f>
+        <v>1789845</v>
+      </c>
+      <c r="M12" s="6"/>
+      <c r="N12" s="7">
+        <f ca="1">C12+E12+G12+J12+L12</f>
+        <v>1854950</v>
+      </c>
+      <c r="O12" s="43">
+        <f ca="1">N12/$N$21</f>
+        <v>0.10000001078196294</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="12">
+        <f>SUM(C8:C12)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D13" s="3">
+        <f>SUM(D8:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="8">
+        <f>SUM(E8:E12)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="12">
+        <f>SUM(G8:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
+        <f>SUM(I8:I12)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="8">
+        <f>SUM(J8:J12)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="3"/>
+      <c r="L13" s="12">
+        <f ca="1">SUM(L8:L12)</f>
+        <v>1789845</v>
+      </c>
+      <c r="M13" s="3"/>
+      <c r="N13" s="12">
+        <f ca="1">SUM(N8:N12)</f>
+        <v>11530108</v>
+      </c>
+      <c r="O13" s="56">
+        <f ca="1">N13/$N$21</f>
+        <v>0.62158598577708135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="43"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="9">
+        <f>PreA!D17</f>
+        <v>8000000</v>
+      </c>
+      <c r="E15" s="7">
+        <f>IFERROR(ROUND(D15/$E$22,0),0)</f>
+        <v>1939567</v>
+      </c>
+      <c r="F15" s="6"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="21">
+        <v>5000000</v>
+      </c>
+      <c r="J15" s="7">
+        <f ca="1">IFERROR(ROUND(I15/$J$22,0),0)</f>
+        <v>1159340</v>
+      </c>
+      <c r="K15" s="6"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="7">
+        <f ca="1">C15+E15+G15+J15+L15</f>
+        <v>3098907</v>
+      </c>
+      <c r="O15" s="43">
+        <f ca="1">N15/$N$21</f>
+        <v>0.16706150214954604</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="7"/>
+      <c r="D16" s="9">
+        <f>PreA!D18</f>
+        <v>1825000</v>
+      </c>
+      <c r="E16" s="7">
+        <f>IFERROR(ROUND(D16/$E$22,0),0)</f>
+        <v>442464</v>
+      </c>
+      <c r="F16" s="6"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="7">
+        <f>C16+E16+G16+J16+L16</f>
+        <v>442464</v>
+      </c>
+      <c r="O16" s="43">
+        <f ca="1">N16/$N$21</f>
+        <v>2.3853152252422141E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="21">
+        <v>12000000</v>
+      </c>
+      <c r="J17" s="7">
+        <f ca="1">IFERROR(ROUND(I17/$J$22,0),0)</f>
+        <v>2782415</v>
+      </c>
+      <c r="K17" s="6"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="7">
+        <f ca="1">C17+E17+G17+J17+L17</f>
+        <v>2782415</v>
+      </c>
+      <c r="O17" s="43">
+        <f ca="1">N17/$N$21</f>
+        <v>0.14999947707479738</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="10">
+        <f>I21-I15-I17</f>
+        <v>3000000</v>
+      </c>
+      <c r="J18" s="7">
+        <f ca="1">IFERROR(ROUND(I18/$J$22,0),0)</f>
+        <v>695604</v>
+      </c>
+      <c r="K18" s="6"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="7">
+        <f ca="1">C18+E18+G18+J18+L18</f>
+        <v>695604</v>
+      </c>
+      <c r="O18" s="43">
+        <f ca="1">N18/$N$21</f>
+        <v>3.749988274615302E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="43"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="43"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="13">
+        <f>C13+SUM(C15:C18)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D21" s="14">
+        <f>D13+SUM(D15:D18)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E21" s="13">
+        <f>E13+SUM(E15:E18)</f>
+        <v>2382031</v>
+      </c>
+      <c r="F21" s="15"/>
+      <c r="G21" s="13">
+        <f>G13+SUM(G15:G18)</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="15"/>
+      <c r="I21" s="57">
+        <v>20000000</v>
+      </c>
+      <c r="J21" s="13">
+        <f ca="1">SUM(J15:J18)</f>
+        <v>4637359</v>
+      </c>
+      <c r="K21" s="15"/>
+      <c r="L21" s="13">
+        <f ca="1">L13+SUM(L15:L18)</f>
+        <v>1789845</v>
+      </c>
+      <c r="M21" s="15"/>
+      <c r="N21" s="13">
+        <f ca="1">N13+SUM(N15:N18)</f>
+        <v>18549498</v>
+      </c>
+      <c r="O21" s="52">
+        <f ca="1">SUM(O13,O15:O18)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="11">
+        <f>(C28-D21)/PreA!F21</f>
+        <v>4.1246319529565065</v>
+      </c>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="11">
+        <f ca="1">IFERROR(ROUND(J23/(C13+E21+L12),4),0)</f>
+        <v>4.3128000000000002</v>
+      </c>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="38"/>
+    </row>
+    <row r="23" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="21">
+        <v>60000000</v>
+      </c>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="38"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="10">
+        <f>J23+I21</f>
+        <v>80000000</v>
+      </c>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="38"/>
+    </row>
+    <row r="25" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1"/>
+      <c r="B25" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="40"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="55">
+        <f ca="1">E21/(E21+C13+L12)</f>
+        <v>0.17121960900476915</v>
+      </c>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="40"/>
+      <c r="J25" s="55">
+        <f ca="1">J21/N21</f>
+        <v>0.24999916439787212</v>
+      </c>
+      <c r="K25" s="40"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="40"/>
+      <c r="N25" s="40"/>
+      <c r="O25" s="41"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+      <c r="B27" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="20">
+        <v>50000000</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="4">
+        <f>J23</f>
+        <v>60000000</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="4">
+        <f>I21</f>
+        <v>20000000</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" s="23">
+        <v>0.1</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="4">
+        <f>I17</f>
+        <v>12000000</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" s="4">
+        <f>I15</f>
+        <v>5000000</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="4">
+        <f>I18</f>
+        <v>3000000</v>
+      </c>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint: Series B fixes: accounting formats, input in assumptions section
</commit_message>
<xml_diff>
--- a/runs/20260414-110202/models/model.xlsx
+++ b/runs/20260414-110202/models/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5988BF2C-0D55-9F4E-B96A-D7ECCC229F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{79731E4C-1106-EF41-943B-B218D84FEA9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="119" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="SAFE Investments" sheetId="122" r:id="rId3"/>
     <sheet name="PreA" sheetId="123" r:id="rId4"/>
     <sheet name="Series A" sheetId="124" r:id="rId5"/>
+    <sheet name="Series B" sheetId="125" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="105">
   <si>
     <t>Total</t>
   </si>
@@ -270,6 +271,21 @@
     <t>SAFE Post-Money Valuation Cap</t>
   </si>
   <si>
+    <t>Series B</t>
+  </si>
+  <si>
+    <t>Pre B</t>
+  </si>
+  <si>
+    <t>Series B Assumptions:</t>
+  </si>
+  <si>
+    <t>% Ownership</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation Step-up</t>
+  </si>
+  <si>
     <t>Common</t>
   </si>
   <si>
@@ -288,6 +304,9 @@
     <t>Other SAFE Investors</t>
   </si>
   <si>
+    <t>Other Series B Investors</t>
+  </si>
+  <si>
     <t>Invested</t>
   </si>
   <si>
@@ -325,16 +344,28 @@
   </si>
   <si>
     <t>Accomplice New Money</t>
+  </si>
+  <si>
+    <t>1011 VENTURES SERIES B</t>
+  </si>
+  <si>
+    <t>% New Money</t>
+  </si>
+  <si>
+    <t>Option Pool (gross % of post-B FD)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="6">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.0000"/>
+    <numFmt numFmtId="169" formatCode="0.0%_);\(0.0%\);0.0%_);@_)"/>
+    <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="27" x14ac:knownFonts="1">
     <font>
@@ -711,7 +742,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -949,6 +980,21 @@
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1032,7 +1078,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1040,6 +1086,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1093,27 +1140,36 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1126,13 +1182,13 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1155,7 +1211,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1176,6 +1232,9 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1183,6 +1242,46 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="25" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="178" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="19" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="25" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="19" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="19" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1604,518 +1703,518 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="16"/>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="A1" s="17"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="16"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="17" t="s">
+      <c r="A2" s="17"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="16"/>
-      <c r="B3" s="17" t="s">
+      <c r="A3" s="17"/>
+      <c r="B3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="H3" s="17" t="s">
+      <c r="G3" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="H3" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16" t="s">
+      <c r="A4" s="17"/>
+      <c r="B4" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="19">
         <v>3600000</v>
       </c>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18">
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="20">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16" t="s">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="19">
         <v>3600000</v>
       </c>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18">
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="20">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
-      <c r="K5" s="16"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16" t="s">
+      <c r="A6" s="17"/>
+      <c r="B6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="19">
         <v>222187</v>
       </c>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18">
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="20">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="16"/>
-      <c r="J6" s="16"/>
-      <c r="K6" s="16"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16" t="s">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="19">
         <v>592500</v>
       </c>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18">
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="20">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16" t="s">
+      <c r="A8" s="17"/>
+      <c r="B8" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="19">
         <v>592500</v>
       </c>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18">
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="20">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16" t="s">
+      <c r="A9" s="17"/>
+      <c r="B9" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="19">
         <v>13500</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <v>98900</v>
       </c>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18">
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="20">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16" t="s">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="19">
         <v>9000</v>
       </c>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18">
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="20">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16" t="s">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18">
+      <c r="C11" s="19"/>
+      <c r="D11" s="19">
         <v>95000</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18">
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="20">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16" t="s">
+      <c r="A12" s="17"/>
+      <c r="B12" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18">
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19">
         <v>25000</v>
       </c>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18">
+      <c r="F12" s="19"/>
+      <c r="G12" s="19">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="20">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="16"/>
-      <c r="J12" s="16"/>
-      <c r="K12" s="16"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16" t="s">
+      <c r="A13" s="17"/>
+      <c r="B13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18">
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19">
         <v>41562</v>
       </c>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18">
+      <c r="F13" s="19"/>
+      <c r="G13" s="19">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="20">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="16"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="16"/>
-      <c r="B14" s="16" t="s">
+      <c r="A14" s="17"/>
+      <c r="B14" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18">
+      <c r="C14" s="19"/>
+      <c r="D14" s="19">
         <v>285000</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18">
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="19">
+      <c r="H14" s="20">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="16"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16" t="s">
+      <c r="A15" s="17"/>
+      <c r="B15" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18">
+      <c r="C15" s="19"/>
+      <c r="D15" s="19">
         <v>50000</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18">
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="19">
+      <c r="H15" s="20">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="16"/>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16" t="s">
+      <c r="A16" s="17"/>
+      <c r="B16" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18">
+      <c r="C16" s="19"/>
+      <c r="D16" s="19">
         <v>285000</v>
       </c>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18">
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="20">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16" t="s">
+      <c r="A17" s="17"/>
+      <c r="B17" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18">
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19">
         <v>96186</v>
       </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18">
+      <c r="F17" s="19"/>
+      <c r="G17" s="19">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="19">
+      <c r="H17" s="20">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="16"/>
-      <c r="B18" s="16" t="s">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18">
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19">
         <v>48095</v>
       </c>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18">
+      <c r="F18" s="19"/>
+      <c r="G18" s="19">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="19">
+      <c r="H18" s="20">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16" t="s">
+      <c r="A19" s="17"/>
+      <c r="B19" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18">
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19">
         <v>12395</v>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="19">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="19">
+      <c r="H19" s="20">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="16"/>
-      <c r="B20" s="16" t="s">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18">
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19">
         <v>8333</v>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="19">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="20">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16" t="s">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18">
+      <c r="C21" s="19"/>
+      <c r="D21" s="19">
         <v>65105</v>
       </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18">
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="20">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="17"/>
+      <c r="K22" s="17"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="16"/>
-      <c r="B23" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23" s="46">
+      <c r="A23" s="17"/>
+      <c r="B23" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="50">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="46">
+      <c r="D23" s="50">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="46">
+      <c r="E23" s="50">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="46">
+      <c r="F23" s="50">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="46">
+      <c r="G23" s="50">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2136,476 +2235,476 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="24"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="A1" s="26"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="24"/>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
+      <c r="A2" s="26"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="24"/>
-      <c r="B3" s="17" t="s">
+      <c r="A3" s="26"/>
+      <c r="B3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="17" t="s">
+      <c r="D3" s="26"/>
+      <c r="E3" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="24"/>
-      <c r="B4" s="16" t="s">
+      <c r="A4" s="26"/>
+      <c r="B4" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="23">
         <v>25000</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16" t="s">
+      <c r="D4" s="17"/>
+      <c r="E4" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="24"/>
-      <c r="B5" s="16" t="s">
+      <c r="A5" s="26"/>
+      <c r="B5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="23">
         <v>25000</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
-      <c r="K5" s="24"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
-      <c r="B6" s="16" t="s">
+      <c r="A6" s="26"/>
+      <c r="B6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="23">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
-      <c r="K6" s="24"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
-      <c r="B7" s="16" t="s">
+      <c r="A7" s="26"/>
+      <c r="B7" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="23">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
-      <c r="B8" s="16" t="s">
+      <c r="A8" s="26"/>
+      <c r="B8" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="23">
         <v>16566</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
-      <c r="K8" s="24"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="26"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
-      <c r="B9" s="16" t="s">
+      <c r="A9" s="26"/>
+      <c r="B9" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C9" s="23">
         <v>250000</v>
       </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="24"/>
-      <c r="B10" s="16" t="s">
+      <c r="A10" s="26"/>
+      <c r="B10" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="23">
         <v>100000</v>
       </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="26"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
-      <c r="B11" s="16" t="s">
+      <c r="A11" s="26"/>
+      <c r="B11" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="23">
         <v>300000</v>
       </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16" t="s">
+      <c r="D11" s="17"/>
+      <c r="E11" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
-      <c r="B12" s="16" t="s">
+      <c r="A12" s="26"/>
+      <c r="B12" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="22">
+      <c r="C12" s="23">
         <v>37500</v>
       </c>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16" t="s">
+      <c r="D12" s="17"/>
+      <c r="E12" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="24"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="24"/>
-      <c r="B13" s="16" t="s">
+      <c r="A13" s="26"/>
+      <c r="B13" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="23">
         <v>250000</v>
       </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="24"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="24"/>
-      <c r="B14" s="16" t="s">
+      <c r="A14" s="26"/>
+      <c r="B14" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="22">
+      <c r="C14" s="23">
         <v>100000</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="24"/>
-      <c r="B15" s="16" t="s">
+      <c r="A15" s="26"/>
+      <c r="B15" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="23">
         <v>41164</v>
       </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="24"/>
-      <c r="B16" s="16" t="s">
+      <c r="A16" s="26"/>
+      <c r="B16" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="23">
         <v>2328778</v>
       </c>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="24"/>
-      <c r="K16" s="24"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="24"/>
-      <c r="B17" s="16" t="s">
+      <c r="A17" s="26"/>
+      <c r="B17" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="23">
         <v>1506000</v>
       </c>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16" t="s">
+      <c r="D17" s="17"/>
+      <c r="E17" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
-      <c r="K17" s="24"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
-      <c r="B18" s="16" t="s">
+      <c r="A18" s="26"/>
+      <c r="B18" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="23">
         <v>50000</v>
       </c>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
-      <c r="K18" s="24"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="26"/>
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="24"/>
-      <c r="B19" s="16" t="s">
+      <c r="A19" s="26"/>
+      <c r="B19" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="22">
+      <c r="C19" s="23">
         <v>212500</v>
       </c>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16" t="s">
+      <c r="D19" s="17"/>
+      <c r="E19" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="26"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="24"/>
-      <c r="B20" s="16" t="s">
+      <c r="A20" s="26"/>
+      <c r="B20" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="23">
         <v>25000</v>
       </c>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="24"/>
-      <c r="B21" s="16" t="s">
+      <c r="A21" s="26"/>
+      <c r="B21" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="23">
         <v>61746</v>
       </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
-      <c r="J21" s="24"/>
-      <c r="K21" s="24"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
-      <c r="B22" s="16" t="s">
+      <c r="A22" s="26"/>
+      <c r="B22" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="23">
         <v>100000</v>
       </c>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
-      <c r="J22" s="24"/>
-      <c r="K22" s="24"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="24"/>
-      <c r="B23" s="16" t="s">
+      <c r="A23" s="26"/>
+      <c r="B23" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23" s="23">
         <v>100000</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
-      <c r="J23" s="24"/>
-      <c r="K23" s="24"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="26"/>
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="24"/>
-      <c r="B24" s="16" t="s">
+      <c r="A24" s="26"/>
+      <c r="B24" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="23">
         <v>61746</v>
       </c>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
-      <c r="J24" s="24"/>
-      <c r="K24" s="24"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="26"/>
+      <c r="I24" s="26"/>
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="24"/>
-      <c r="B25" s="16" t="s">
+      <c r="A25" s="26"/>
+      <c r="B25" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="22">
+      <c r="C25" s="23">
         <v>250000</v>
       </c>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16" t="s">
+      <c r="D25" s="17"/>
+      <c r="E25" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="24"/>
-      <c r="K25" s="24"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="26"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="26"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="24"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
-      <c r="K26" s="24"/>
+      <c r="A26" s="26"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="26"/>
+      <c r="J26" s="26"/>
+      <c r="K26" s="26"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="24"/>
-      <c r="B27" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" s="22">
+      <c r="A27" s="26"/>
+      <c r="B27" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="23">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
-      <c r="J27" s="24"/>
-      <c r="K27" s="24"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2655,294 +2754,294 @@
     </row>
     <row r="4" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
-      <c r="B4" s="25" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
+      <c r="B4" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
     </row>
     <row r="5" spans="1:7" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
+      <c r="B5" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="6" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D6" s="31" t="s">
+      <c r="C6" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="29" t="s">
+      <c r="E6" s="7"/>
+      <c r="F6" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="39"/>
+      <c r="G6" s="43"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="40" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="36" t="s">
+      <c r="E7" s="7"/>
+      <c r="F7" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="53" t="s">
+      <c r="G7" s="57" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="D8" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="30" t="s">
+      <c r="D8" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="54" t="s">
+      <c r="G8" s="58" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="38"/>
+      <c r="C9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="42"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="6">
         <f>'Detailed Cap Table'!C4</f>
         <v>3600000</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="7">
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="8">
         <f>C10</f>
         <v>3600000</v>
       </c>
-      <c r="G10" s="43">
+      <c r="G10" s="47">
         <f>F10/$F$21</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="6">
         <f>'Detailed Cap Table'!C5</f>
         <v>3600000</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="7">
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="8">
         <f>C11</f>
         <v>3600000</v>
       </c>
-      <c r="G11" s="43">
+      <c r="G11" s="47">
         <f>F11/$F$21</f>
         <v>0.36959987630724139</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="C12" s="5">
+      <c r="B12" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="6">
         <f>'Detailed Cap Table'!C6+'Detailed Cap Table'!C7+'Detailed Cap Table'!C8+'Detailed Cap Table'!C9+'Detailed Cap Table'!C10+'Detailed Cap Table'!F19+'Detailed Cap Table'!F20</f>
         <v>1450415</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="7">
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="8">
         <f>C12</f>
         <v>1450415</v>
       </c>
-      <c r="G12" s="43">
+      <c r="G12" s="47">
         <f>F12/$F$21</f>
         <v>0.14890922349837987</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="5">
+      <c r="B13" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" s="6">
         <f>SUM('Detailed Cap Table'!D4:D20)+SUM('Detailed Cap Table'!E4:E20)</f>
         <v>1024743</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7">
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="8">
         <f>C13</f>
         <v>1024743</v>
       </c>
-      <c r="G13" s="43">
+      <c r="G13" s="47">
         <f>F13/$F$21</f>
         <v>0.10520691279075318</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="49">
+      <c r="B14" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="53">
         <f>'Detailed Cap Table'!D21</f>
         <v>65105</v>
       </c>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="50">
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="54">
         <f>C14</f>
         <v>65105</v>
       </c>
-      <c r="G14" s="51">
+      <c r="G14" s="55">
         <f>F14/$F$21</f>
         <v>6.6841110963841528E-3</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="9">
         <f>SUM(C10:C14)</f>
         <v>9740263</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
-      <c r="F15" s="8">
+      <c r="F15" s="9">
         <f>SUM(F10:F14)</f>
         <v>9740263</v>
       </c>
-      <c r="G15" s="44">
+      <c r="G15" s="48">
         <f>SUM(G10:G14)</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="43"/>
+      <c r="B16" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="47"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="9">
+      <c r="C17" s="8"/>
+      <c r="D17" s="10">
         <f>'SAFE Investments'!C6+'SAFE Investments'!C7+'SAFE Investments'!C8+'SAFE Investments'!C15+'SAFE Investments'!C16+'SAFE Investments'!C17+'SAFE Investments'!C21+'SAFE Investments'!C24</f>
         <v>8000000</v>
       </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="7">
+      <c r="E17" s="7"/>
+      <c r="F17" s="8">
         <f>C17</f>
         <v>0</v>
       </c>
-      <c r="G17" s="43">
+      <c r="G17" s="47">
         <f>F17/$F$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="9">
+      <c r="B18" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="8"/>
+      <c r="D18" s="10">
         <f>'SAFE Investments'!C27-D17</f>
         <v>1825000</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="7">
+      <c r="E18" s="7"/>
+      <c r="F18" s="8">
         <f>C18</f>
         <v>0</v>
       </c>
-      <c r="G18" s="43">
+      <c r="G18" s="47">
         <f>F18/$F$21</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="43"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="47"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="43"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="47"/>
     </row>
     <row r="21" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="45" t="s">
+      <c r="B21" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="14">
         <f>C15</f>
         <v>9740263</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="15">
         <f>SUM(D17:D18)</f>
         <v>9825000</v>
       </c>
-      <c r="E21" s="15"/>
-      <c r="F21" s="13">
+      <c r="E21" s="16"/>
+      <c r="F21" s="14">
         <f>F15</f>
         <v>9740263</v>
       </c>
-      <c r="G21" s="52">
+      <c r="G21" s="56">
         <f>SUM(G10:G14)</f>
         <v>1</v>
       </c>
@@ -2950,52 +3049,52 @@
     <row r="22" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
     </row>
     <row r="23" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C23" s="11">
+        <v>95</v>
+      </c>
+      <c r="C23" s="12">
         <f>D24/C25</f>
         <v>5.1333316153783528</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="21">
+      <c r="C24" s="7"/>
+      <c r="D24" s="22">
         <v>50000000</v>
       </c>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
     </row>
     <row r="25" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C25" s="7">
+        <v>96</v>
+      </c>
+      <c r="C25" s="8">
         <f>F21</f>
         <v>9740263</v>
       </c>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
@@ -3071,40 +3170,40 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
+      <c r="B1" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
       <c r="O1" s="1"/>
     </row>
     <row r="2" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
+      <c r="B2" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -3127,269 +3226,269 @@
     <row r="4" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" s="31" t="s">
+      <c r="C4" s="33" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="39"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="29" t="s">
+      <c r="E4" s="43"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="39"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="31" t="s">
-        <v>78</v>
-      </c>
-      <c r="M4" s="6"/>
-      <c r="N4" s="29" t="s">
+      <c r="J4" s="43"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="M4" s="7"/>
+      <c r="N4" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="O4" s="39"/>
+      <c r="O4" s="43"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="37" t="s">
+      <c r="F5" s="7"/>
+      <c r="G5" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="29" t="s">
+      <c r="H5" s="7"/>
+      <c r="I5" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="J5" s="39" t="s">
+      <c r="J5" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="37" t="s">
+      <c r="K5" s="7"/>
+      <c r="L5" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="M5" s="6"/>
-      <c r="N5" s="29" t="s">
+      <c r="M5" s="7"/>
+      <c r="N5" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="O5" s="39" t="s">
+      <c r="O5" s="43" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="36" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="53" t="s">
+      <c r="D6" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" s="57" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="37" t="s">
-        <v>79</v>
-      </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="36" t="s">
-        <v>83</v>
-      </c>
-      <c r="J6" s="53" t="s">
+      <c r="F6" s="7"/>
+      <c r="G6" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="7"/>
+      <c r="I6" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="J6" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="6"/>
-      <c r="L6" s="37" t="s">
+      <c r="K6" s="7"/>
+      <c r="L6" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="M6" s="6"/>
-      <c r="N6" s="36" t="s">
+      <c r="M6" s="7"/>
+      <c r="N6" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="O6" s="53" t="s">
+      <c r="O6" s="57" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="33"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
-      <c r="N7" s="33"/>
-      <c r="O7" s="48"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="37"/>
+      <c r="M7" s="37"/>
+      <c r="N7" s="37"/>
+      <c r="O7" s="52"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="6">
         <f>PreA!C10</f>
         <v>3600000</v>
       </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="7">
+      <c r="D8" s="7"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="8">
         <f>C8+E8+G8+J8+L8</f>
         <v>3600000</v>
       </c>
-      <c r="O8" s="43">
+      <c r="O8" s="47">
         <f ca="1">N8/$N$21</f>
         <v>0.19407533292814716</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="6">
         <f>PreA!C11</f>
         <v>3600000</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="7">
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="8">
         <f>C9+E9+G9+J9+L9</f>
         <v>3600000</v>
       </c>
-      <c r="O9" s="43">
+      <c r="O9" s="47">
         <f ca="1">N9/$N$21</f>
         <v>0.19407533292814716</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="5">
+      <c r="B10" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="6">
         <f>PreA!C12</f>
         <v>1450415</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="7">
+      <c r="D10" s="7"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="8">
         <f>C10+E10+G10+J10+L10</f>
         <v>1450415</v>
       </c>
-      <c r="O10" s="43">
+      <c r="O10" s="47">
         <f ca="1">N10/$N$21</f>
         <v>7.8191603891382938E-2</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="C11" s="5">
+      <c r="B11" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="6">
         <f>PreA!C13</f>
         <v>1024743</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="7">
+      <c r="D11" s="7"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="8">
         <f>C11+E11+G11+J11+L11</f>
         <v>1024743</v>
       </c>
-      <c r="O11" s="43">
+      <c r="O11" s="47">
         <f ca="1">N11/$N$21</f>
         <v>5.5243705247441197E-2</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="C12" s="5">
+      <c r="B12" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="6">
         <f>PreA!C14</f>
         <v>65105</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="7">
+      <c r="D12" s="7"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="8">
         <f ca="1">ROUND((C31*(C13+E21+J21)-C12)/(1-C31),0)</f>
         <v>1789845</v>
       </c>
-      <c r="M12" s="6"/>
-      <c r="N12" s="7">
+      <c r="M12" s="7"/>
+      <c r="N12" s="8">
         <f ca="1">C12+E12+G12+J12+L12</f>
         <v>1854950</v>
       </c>
-      <c r="O12" s="43">
+      <c r="O12" s="47">
         <f ca="1">N12/$N$21</f>
         <v>0.10000001078196294</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="27" t="s">
+      <c r="B13" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="13">
         <f>SUM(C8:C12)</f>
         <v>9740263</v>
       </c>
@@ -3397,12 +3496,12 @@
         <f>SUM(D8:D12)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="9">
         <f>SUM(E8:E12)</f>
         <v>0</v>
       </c>
       <c r="F13" s="3"/>
-      <c r="G13" s="12">
+      <c r="G13" s="13">
         <f>SUM(G8:G12)</f>
         <v>0</v>
       </c>
@@ -3411,343 +3510,343 @@
         <f>SUM(I8:I12)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="9">
         <f>SUM(J8:J12)</f>
         <v>0</v>
       </c>
       <c r="K13" s="3"/>
-      <c r="L13" s="12">
+      <c r="L13" s="13">
         <f ca="1">SUM(L8:L12)</f>
         <v>1789845</v>
       </c>
       <c r="M13" s="3"/>
-      <c r="N13" s="12">
+      <c r="N13" s="13">
         <f ca="1">SUM(N8:N12)</f>
         <v>11530108</v>
       </c>
-      <c r="O13" s="56">
+      <c r="O13" s="61">
         <f ca="1">N13/$N$21</f>
         <v>0.62158598577708135</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="43"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="47"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="9">
+      <c r="C15" s="8"/>
+      <c r="D15" s="10">
         <f>PreA!D17</f>
         <v>8000000</v>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="8">
         <f>IFERROR(ROUND(D15/$E$22,0),0)</f>
         <v>1939567</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="21">
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="22">
         <v>5000000</v>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="8">
         <f ca="1">IFERROR(ROUND(I15/$J$22,0),0)</f>
         <v>1159340</v>
       </c>
-      <c r="K15" s="6"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="7">
+      <c r="K15" s="7"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="8">
         <f ca="1">C15+E15+G15+J15+L15</f>
         <v>3098907</v>
       </c>
-      <c r="O15" s="43">
+      <c r="O15" s="47">
         <f ca="1">N15/$N$21</f>
         <v>0.16706150214954604</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="9">
+      <c r="B16" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="10">
         <f>PreA!D18</f>
         <v>1825000</v>
       </c>
-      <c r="E16" s="7">
+      <c r="E16" s="8">
         <f>IFERROR(ROUND(D16/$E$22,0),0)</f>
         <v>442464</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="7">
+      <c r="F16" s="7"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="8">
         <f>C16+E16+G16+J16+L16</f>
         <v>442464</v>
       </c>
-      <c r="O16" s="43">
+      <c r="O16" s="47">
         <f ca="1">N16/$N$21</f>
         <v>2.3853152252422141E-2</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="26" t="s">
+      <c r="B17" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="21">
+      <c r="C17" s="8"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="22">
         <v>12000000</v>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="8">
         <f ca="1">IFERROR(ROUND(I17/$J$22,0),0)</f>
         <v>2782415</v>
       </c>
-      <c r="K17" s="6"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="7">
+      <c r="K17" s="7"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="8">
         <f ca="1">C17+E17+G17+J17+L17</f>
         <v>2782415</v>
       </c>
-      <c r="O17" s="43">
+      <c r="O17" s="47">
         <f ca="1">N17/$N$21</f>
         <v>0.14999947707479738</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="10">
+      <c r="C18" s="8"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="11">
         <f>I21-I15-I17</f>
         <v>3000000</v>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="8">
         <f ca="1">IFERROR(ROUND(I18/$J$22,0),0)</f>
         <v>695604</v>
       </c>
-      <c r="K18" s="6"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="7">
+      <c r="K18" s="7"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="8">
         <f ca="1">C18+E18+G18+J18+L18</f>
         <v>695604</v>
       </c>
-      <c r="O18" s="43">
+      <c r="O18" s="47">
         <f ca="1">N18/$N$21</f>
         <v>3.749988274615302E-2</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="7"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="43"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="47"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="7"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="43"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="47"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="14">
         <f>C13+SUM(C15:C18)</f>
         <v>9740263</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="15">
         <f>D13+SUM(D15:D18)</f>
         <v>9825000</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="14">
         <f>E13+SUM(E15:E18)</f>
         <v>2382031</v>
       </c>
-      <c r="F21" s="15"/>
-      <c r="G21" s="13">
+      <c r="F21" s="16"/>
+      <c r="G21" s="14">
         <f>G13+SUM(G15:G18)</f>
         <v>0</v>
       </c>
-      <c r="H21" s="15"/>
-      <c r="I21" s="57">
+      <c r="H21" s="16"/>
+      <c r="I21" s="62">
         <v>20000000</v>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="14">
         <f ca="1">SUM(J15:J18)</f>
         <v>4637359</v>
       </c>
-      <c r="K21" s="15"/>
-      <c r="L21" s="13">
+      <c r="K21" s="16"/>
+      <c r="L21" s="14">
         <f ca="1">L13+SUM(L15:L18)</f>
         <v>1789845</v>
       </c>
-      <c r="M21" s="15"/>
-      <c r="N21" s="13">
+      <c r="M21" s="16"/>
+      <c r="N21" s="14">
         <f ca="1">N13+SUM(N15:N18)</f>
         <v>18549498</v>
       </c>
-      <c r="O21" s="52">
+      <c r="O21" s="56">
         <f ca="1">SUM(O13,O15:O18)</f>
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="11">
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="12">
         <f>(C28-D21)/PreA!F21</f>
         <v>4.1246319529565065</v>
       </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="11">
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="12">
         <f ca="1">IFERROR(ROUND(J23/(C13+E21+L12),4),0)</f>
         <v>4.3128000000000002</v>
       </c>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="38"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
+      <c r="O22" s="42"/>
     </row>
     <row r="23" spans="1:15" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="21">
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="22">
         <v>60000000</v>
       </c>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
-      <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="38"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="42"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="10">
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="11">
         <f>J23+I21</f>
         <v>80000000</v>
       </c>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="38"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
+      <c r="N24" s="7"/>
+      <c r="O24" s="42"/>
     </row>
     <row r="25" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="55">
+      <c r="B25" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="60">
         <f ca="1">E21/(E21+C13+L12)</f>
         <v>0.17121960900476915</v>
       </c>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40"/>
-      <c r="J25" s="55">
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="60">
         <f ca="1">J21/N21</f>
         <v>0.24999916439787212</v>
       </c>
-      <c r="K25" s="40"/>
-      <c r="L25" s="40"/>
-      <c r="M25" s="40"/>
-      <c r="N25" s="40"/>
-      <c r="O25" s="41"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="44"/>
+      <c r="M25" s="44"/>
+      <c r="N25" s="44"/>
+      <c r="O25" s="45"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
@@ -3790,7 +3889,7 @@
       <c r="B28" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="21">
         <v>50000000</v>
       </c>
       <c r="D28" s="1"/>
@@ -3853,9 +3952,9 @@
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C31" s="23">
+        <v>100</v>
+      </c>
+      <c r="C31" s="24">
         <v>0.1</v>
       </c>
       <c r="D31" s="1"/>
@@ -3896,7 +3995,7 @@
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C33" s="4">
         <f>I15</f>
@@ -3957,4 +4056,1381 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D507087C-AF9C-134D-862F-ACFABDF57E2D}">
+  <dimension ref="A1:T40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="33.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="10" max="10" width="15.5" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="15.5" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="0.5" customWidth="1"/>
+    <col min="17" max="17" width="11.83203125" customWidth="1"/>
+    <col min="18" max="18" width="0.5" customWidth="1"/>
+    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27"/>
+      <c r="T1" s="1"/>
+    </row>
+    <row r="2" spans="1:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="27"/>
+      <c r="T2" s="1"/>
+    </row>
+    <row r="3" spans="1:20" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+    </row>
+    <row r="4" spans="1:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="59" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="43"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="H4" s="3"/>
+      <c r="I4" s="59" t="s">
+        <v>52</v>
+      </c>
+      <c r="J4" s="43"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="M4" s="3"/>
+      <c r="N4" s="59" t="s">
+        <v>77</v>
+      </c>
+      <c r="O4" s="43"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="R4" s="3"/>
+      <c r="S4" s="59" t="s">
+        <v>53</v>
+      </c>
+      <c r="T4" s="43"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="3"/>
+      <c r="L5" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="M5" s="3"/>
+      <c r="N5" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="O5" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="R5" s="3"/>
+      <c r="S5" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="T5" s="43" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" s="57" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="41" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="J6" s="57" t="s">
+        <v>60</v>
+      </c>
+      <c r="K6" s="3"/>
+      <c r="L6" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="3"/>
+      <c r="N6" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="O6" s="57" t="s">
+        <v>60</v>
+      </c>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="41" t="s">
+        <v>78</v>
+      </c>
+      <c r="R6" s="3"/>
+      <c r="S6" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="T6" s="57" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="51" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="37"/>
+      <c r="M7" s="37"/>
+      <c r="N7" s="37"/>
+      <c r="O7" s="37"/>
+      <c r="P7" s="37"/>
+      <c r="Q7" s="37"/>
+      <c r="R7" s="37"/>
+      <c r="S7" s="37"/>
+      <c r="T7" s="52"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="29" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="64">
+        <f>'Series A'!C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="D8" s="69"/>
+      <c r="E8" s="64">
+        <f>'Series A'!E8</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="64">
+        <f>'Series A'!G8</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="7"/>
+      <c r="I8" s="69"/>
+      <c r="J8" s="64">
+        <f>'Series A'!J8</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="7"/>
+      <c r="L8" s="64">
+        <f>'Series A'!L8</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="7"/>
+      <c r="N8" s="71"/>
+      <c r="O8" s="66"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="66"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="66">
+        <f>C8+E8+G8+J8+L8+O8+Q8</f>
+        <v>3600000</v>
+      </c>
+      <c r="T8" s="32">
+        <f ca="1">S8/$S$22</f>
+        <v>0.14814413667317156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="64">
+        <f>'Series A'!C9</f>
+        <v>3600000</v>
+      </c>
+      <c r="D9" s="69"/>
+      <c r="E9" s="64">
+        <f>'Series A'!E9</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="G9" s="64">
+        <f>'Series A'!G9</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="7"/>
+      <c r="I9" s="69"/>
+      <c r="J9" s="64">
+        <f>'Series A'!J9</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="7"/>
+      <c r="L9" s="64">
+        <f>'Series A'!L9</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="7"/>
+      <c r="N9" s="71"/>
+      <c r="O9" s="66"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="66"/>
+      <c r="R9" s="7"/>
+      <c r="S9" s="66">
+        <f>C9+E9+G9+J9+L9+O9+Q9</f>
+        <v>3600000</v>
+      </c>
+      <c r="T9" s="32">
+        <f ca="1">S9/$S$22</f>
+        <v>0.14814413667317156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="64">
+        <f>'Series A'!C10</f>
+        <v>1450415</v>
+      </c>
+      <c r="D10" s="69"/>
+      <c r="E10" s="64">
+        <f>'Series A'!E10</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="G10" s="64">
+        <f>'Series A'!G10</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="7"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="64">
+        <f>'Series A'!J10</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="7"/>
+      <c r="L10" s="64">
+        <f>'Series A'!L10</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="7"/>
+      <c r="N10" s="71"/>
+      <c r="O10" s="66"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="66"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="66">
+        <f>C10+E10+G10+J10+L10+O10+Q10</f>
+        <v>1450415</v>
+      </c>
+      <c r="T10" s="32">
+        <f ca="1">S10/$S$22</f>
+        <v>5.9686243886893926E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="C11" s="64">
+        <f>'Series A'!C11</f>
+        <v>1024743</v>
+      </c>
+      <c r="D11" s="69"/>
+      <c r="E11" s="64">
+        <f>'Series A'!E11</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="64">
+        <f>'Series A'!G11</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="7"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="64">
+        <f>'Series A'!J11</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="7"/>
+      <c r="L11" s="64">
+        <f>'Series A'!L11</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="7"/>
+      <c r="N11" s="71"/>
+      <c r="O11" s="66"/>
+      <c r="P11" s="7"/>
+      <c r="Q11" s="66"/>
+      <c r="R11" s="7"/>
+      <c r="S11" s="66">
+        <f>C11+E11+G11+J11+L11+O11+Q11</f>
+        <v>1024743</v>
+      </c>
+      <c r="T11" s="32">
+        <f ca="1">S11/$S$22</f>
+        <v>4.2169351957465517E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="C12" s="64">
+        <f>'Series A'!C12</f>
+        <v>65105</v>
+      </c>
+      <c r="D12" s="69"/>
+      <c r="E12" s="64">
+        <f>'Series A'!E12</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="7"/>
+      <c r="G12" s="64">
+        <f>'Series A'!G12</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="7"/>
+      <c r="I12" s="69"/>
+      <c r="J12" s="64">
+        <f>'Series A'!J12</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="7"/>
+      <c r="L12" s="64">
+        <f ca="1">'Series A'!L12</f>
+        <v>1789845</v>
+      </c>
+      <c r="M12" s="7"/>
+      <c r="N12" s="71"/>
+      <c r="O12" s="66"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="66">
+        <f ca="1">ROUND(C34*S22,0)</f>
+        <v>1701046</v>
+      </c>
+      <c r="R12" s="7"/>
+      <c r="S12" s="66">
+        <f ca="1">C12+E12+G12+J12+L12+O12+Q12</f>
+        <v>3555996</v>
+      </c>
+      <c r="T12" s="32">
+        <f ca="1">S12/$S$22</f>
+        <v>0.1463333215092365</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="65">
+        <f>SUM(C8:C12)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D13" s="70">
+        <f>SUM(D8:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="68">
+        <f>SUM(E8:E12)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="3"/>
+      <c r="G13" s="68">
+        <f>SUM(G8:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="3"/>
+      <c r="I13" s="70">
+        <f>SUM(I8:I12)</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="68">
+        <f>SUM(J8:J12)</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="3"/>
+      <c r="L13" s="68">
+        <f ca="1">SUM(L8:L12)</f>
+        <v>1789845</v>
+      </c>
+      <c r="M13" s="3"/>
+      <c r="N13" s="70">
+        <f>SUM(N8:N12)</f>
+        <v>0</v>
+      </c>
+      <c r="O13" s="68">
+        <f>SUM(O8:O12)</f>
+        <v>0</v>
+      </c>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="68">
+        <f ca="1">SUM(Q8:Q12)</f>
+        <v>1701046</v>
+      </c>
+      <c r="R13" s="3"/>
+      <c r="S13" s="68">
+        <f ca="1">SUM(S8:S12)</f>
+        <v>13231154</v>
+      </c>
+      <c r="T13" s="75">
+        <f ca="1">S13/$S$22</f>
+        <v>0.54447719069993905</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="66"/>
+      <c r="D14" s="71"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="66"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="71"/>
+      <c r="J14" s="66"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="66"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="71"/>
+      <c r="O14" s="66"/>
+      <c r="P14" s="7"/>
+      <c r="Q14" s="66"/>
+      <c r="R14" s="7"/>
+      <c r="S14" s="66"/>
+      <c r="T14" s="32"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="64">
+        <f>'Series A'!C15</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="72">
+        <f>'Series A'!D15</f>
+        <v>8000000</v>
+      </c>
+      <c r="E15" s="64">
+        <f>'Series A'!E15</f>
+        <v>1939567</v>
+      </c>
+      <c r="F15" s="7"/>
+      <c r="G15" s="64">
+        <f>'Series A'!G15</f>
+        <v>0</v>
+      </c>
+      <c r="H15" s="7"/>
+      <c r="I15" s="72">
+        <f>'Series A'!I15</f>
+        <v>5000000</v>
+      </c>
+      <c r="J15" s="64">
+        <f ca="1">'Series A'!J15</f>
+        <v>1159340</v>
+      </c>
+      <c r="K15" s="7"/>
+      <c r="L15" s="64">
+        <f>'Series A'!L15</f>
+        <v>0</v>
+      </c>
+      <c r="M15" s="7"/>
+      <c r="N15" s="71">
+        <f ca="1">N22*(1-C33)*('Series A'!E15+'Series A'!J15)/('Series A'!E21+'Series A'!J21)</f>
+        <v>6622171.5847103521</v>
+      </c>
+      <c r="O15" s="66">
+        <f ca="1">IFERROR(ROUND(N15/$O$24,0),0)</f>
+        <v>894018</v>
+      </c>
+      <c r="P15" s="7"/>
+      <c r="Q15" s="66"/>
+      <c r="R15" s="7"/>
+      <c r="S15" s="66">
+        <f ca="1">C15+E15+G15+J15+L15+O15+Q15</f>
+        <v>3992925</v>
+      </c>
+      <c r="T15" s="32">
+        <f ca="1">S15/$S$22</f>
+        <v>0.16431345192381211</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="64">
+        <f>'Series A'!C16</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="72">
+        <f>'Series A'!D16</f>
+        <v>1825000</v>
+      </c>
+      <c r="E16" s="64">
+        <f>'Series A'!E16</f>
+        <v>442464</v>
+      </c>
+      <c r="F16" s="7"/>
+      <c r="G16" s="64">
+        <f>'Series A'!G16</f>
+        <v>0</v>
+      </c>
+      <c r="H16" s="7"/>
+      <c r="I16" s="72">
+        <f>'Series A'!I16</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="64">
+        <f>'Series A'!J16</f>
+        <v>0</v>
+      </c>
+      <c r="K16" s="7"/>
+      <c r="L16" s="64">
+        <f>'Series A'!L16</f>
+        <v>0</v>
+      </c>
+      <c r="M16" s="7"/>
+      <c r="N16" s="71">
+        <f ca="1">N22*(1-C33)*('Series A'!E16+'Series A'!J16)/('Series A'!E21+'Series A'!J21)</f>
+        <v>945518.05783693457</v>
+      </c>
+      <c r="O16" s="66">
+        <f ca="1">IFERROR(ROUND(N16/$O$24,0),0)</f>
+        <v>127649</v>
+      </c>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="66"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="66">
+        <f ca="1">C16+E16+G16+J16+L16+O16+Q16</f>
+        <v>570113</v>
+      </c>
+      <c r="T16" s="32">
+        <f ca="1">S16/$S$22</f>
+        <v>2.3460805053097739E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="64">
+        <f>'Series A'!C17</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="72">
+        <f>'Series A'!D17</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="64">
+        <f>'Series A'!E17</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="7"/>
+      <c r="G17" s="64">
+        <f>'Series A'!G17</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="7"/>
+      <c r="I17" s="72">
+        <f>'Series A'!I17</f>
+        <v>12000000</v>
+      </c>
+      <c r="J17" s="64">
+        <f ca="1">'Series A'!J17</f>
+        <v>2782415</v>
+      </c>
+      <c r="K17" s="7"/>
+      <c r="L17" s="64">
+        <f>'Series A'!L17</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="7"/>
+      <c r="N17" s="71">
+        <f ca="1">N22*(1-C33)*('Series A'!J17)/('Series A'!E21+'Series A'!J21)</f>
+        <v>5945847.8585746055</v>
+      </c>
+      <c r="O17" s="66">
+        <f ca="1">IFERROR(ROUND(N17/$O$24,0),0)</f>
+        <v>802712</v>
+      </c>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="66"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="66">
+        <f ca="1">C17+E17+G17+J17+L17+O17+Q17</f>
+        <v>3585127</v>
+      </c>
+      <c r="T17" s="32">
+        <f ca="1">S17/$S$22</f>
+        <v>0.14753209563296599</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="29" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="64">
+        <f>'Series A'!C18</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="72">
+        <f>'Series A'!D18</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="64">
+        <f>'Series A'!E18</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="7"/>
+      <c r="G18" s="64">
+        <f>'Series A'!G18</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="7"/>
+      <c r="I18" s="72">
+        <f>'Series A'!I18</f>
+        <v>3000000</v>
+      </c>
+      <c r="J18" s="64">
+        <f ca="1">'Series A'!J18</f>
+        <v>695604</v>
+      </c>
+      <c r="K18" s="7"/>
+      <c r="L18" s="64">
+        <f>'Series A'!L18</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="7"/>
+      <c r="N18" s="71">
+        <f ca="1">N22*(1-C33)*('Series A'!J18)/('Series A'!E21+'Series A'!J21)</f>
+        <v>1486462.4988781076</v>
+      </c>
+      <c r="O18" s="66">
+        <f ca="1">IFERROR(ROUND(N18/$O$24,0),0)</f>
+        <v>200678</v>
+      </c>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="66"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="66">
+        <f ca="1">C18+E18+G18+J18+L18+O18+Q18</f>
+        <v>896282</v>
+      </c>
+      <c r="T18" s="32">
+        <f ca="1">S18/$S$22</f>
+        <v>3.6883034196028765E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="66"/>
+      <c r="D19" s="71"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="66"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="71"/>
+      <c r="J19" s="66"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="66"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="71">
+        <f>N22*C33</f>
+        <v>15000000</v>
+      </c>
+      <c r="O19" s="66">
+        <f ca="1">IFERROR(ROUND(N19/$O$24,0),0)</f>
+        <v>2025057</v>
+      </c>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="66"/>
+      <c r="R19" s="7"/>
+      <c r="S19" s="66">
+        <f ca="1">C19+E19+G19+J19+L19+O19+Q19</f>
+        <v>2025057</v>
+      </c>
+      <c r="T19" s="32">
+        <f ca="1">S19/$S$22</f>
+        <v>8.3333422494156331E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="66"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="66"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="71"/>
+      <c r="J20" s="66"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="66"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="69"/>
+      <c r="O20" s="66"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="66"/>
+      <c r="R20" s="7"/>
+      <c r="S20" s="66"/>
+      <c r="T20" s="32"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="66"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="66"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="71"/>
+      <c r="J21" s="66"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="66"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="71"/>
+      <c r="O21" s="66"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="66"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="66"/>
+      <c r="T21" s="32"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="67">
+        <f>C13+SUM(C15:C19)</f>
+        <v>9740263</v>
+      </c>
+      <c r="D22" s="73">
+        <f>D13+SUM(D15:D19)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E22" s="67">
+        <f>E13+SUM(E15:E19)</f>
+        <v>2382031</v>
+      </c>
+      <c r="F22" s="16"/>
+      <c r="G22" s="67">
+        <f>G13+SUM(G15:G19)</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="16"/>
+      <c r="I22" s="73">
+        <f>I13+SUM(I15:I19)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J22" s="67">
+        <f ca="1">J13+SUM(J15:J19)</f>
+        <v>4637359</v>
+      </c>
+      <c r="K22" s="16"/>
+      <c r="L22" s="67">
+        <f ca="1">L13+SUM(L15:L19)</f>
+        <v>1789845</v>
+      </c>
+      <c r="M22" s="16"/>
+      <c r="N22" s="74">
+        <f>C31</f>
+        <v>30000000</v>
+      </c>
+      <c r="O22" s="67">
+        <f ca="1">O13+SUM(O15:O19)</f>
+        <v>4050114</v>
+      </c>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="67">
+        <f ca="1">Q13+SUM(Q15:Q19)</f>
+        <v>1701046</v>
+      </c>
+      <c r="R22" s="16"/>
+      <c r="S22" s="67">
+        <f ca="1">S13+SUM(S15:S19)</f>
+        <v>24300658</v>
+      </c>
+      <c r="T22" s="76">
+        <f ca="1">T13+SUM(T15:T19)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="7"/>
+      <c r="R23" s="7"/>
+      <c r="S23" s="7"/>
+      <c r="T23" s="42"/>
+    </row>
+    <row r="24" spans="1:20" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="29" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12">
+        <f ca="1">'Series A'!J22</f>
+        <v>4.3128000000000002</v>
+      </c>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12">
+        <f ca="1">IFERROR(ROUND(O25/(S22-O22),4),0)</f>
+        <v>7.4071999999999996</v>
+      </c>
+      <c r="P24" s="7"/>
+      <c r="Q24" s="7"/>
+      <c r="R24" s="7"/>
+      <c r="S24" s="7"/>
+      <c r="T24" s="42"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A25" s="1"/>
+      <c r="B25" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11">
+        <f>'Series A'!J23</f>
+        <v>60000000</v>
+      </c>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="22">
+        <v>150000000</v>
+      </c>
+      <c r="P25" s="7"/>
+      <c r="Q25" s="7"/>
+      <c r="R25" s="7"/>
+      <c r="S25" s="7"/>
+      <c r="T25" s="42"/>
+    </row>
+    <row r="26" spans="1:20" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="31" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="63"/>
+      <c r="F26" s="63"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63"/>
+      <c r="I26" s="63"/>
+      <c r="J26" s="63">
+        <f>'Series A'!J24</f>
+        <v>80000000</v>
+      </c>
+      <c r="K26" s="63"/>
+      <c r="L26" s="63"/>
+      <c r="M26" s="63"/>
+      <c r="N26" s="63"/>
+      <c r="O26" s="63">
+        <f>O25+N22</f>
+        <v>180000000</v>
+      </c>
+      <c r="P26" s="44"/>
+      <c r="Q26" s="44"/>
+      <c r="R26" s="44"/>
+      <c r="S26" s="44"/>
+      <c r="T26" s="45"/>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1"/>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
+      <c r="T29" s="1"/>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="5">
+        <f>O25/'Series A'!J24-1</f>
+        <v>0.875</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="21">
+        <v>30000000</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="5">
+        <f>N22/O26</f>
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="24">
+        <v>0.5</v>
+      </c>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="1"/>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" s="24">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1"/>
+      <c r="T34" s="1"/>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
+      <c r="S35" s="1"/>
+      <c r="T35" s="1"/>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1"/>
+      <c r="R36" s="1"/>
+      <c r="S36" s="1"/>
+      <c r="T36" s="1"/>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1"/>
+      <c r="R37" s="1"/>
+      <c r="S37" s="1"/>
+      <c r="T37" s="1"/>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+      <c r="P38" s="1"/>
+      <c r="Q38" s="1"/>
+      <c r="R38" s="1"/>
+      <c r="S38" s="1"/>
+      <c r="T38" s="1"/>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="1"/>
+      <c r="Q39" s="1"/>
+      <c r="R39" s="1"/>
+      <c r="S39" s="1"/>
+      <c r="T39" s="1"/>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="1"/>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1"/>
+      <c r="P40" s="1"/>
+      <c r="Q40" s="1"/>
+      <c r="R40" s="1"/>
+      <c r="S40" s="1"/>
+      <c r="T40" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Checkpoint: Post B Returns sheet built with 3-class waterfall and 1011 returns
</commit_message>
<xml_diff>
--- a/runs/20260414-110202/models/model.xlsx
+++ b/runs/20260414-110202/models/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0A471E57-457E-7842-BD24-C28B4BE8C0F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C033F13-9BEC-7D45-90A9-C61C018C1633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="119" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Series A" sheetId="124" r:id="rId5"/>
     <sheet name="Series B" sheetId="125" r:id="rId6"/>
     <sheet name="Post A Returns" sheetId="126" r:id="rId7"/>
+    <sheet name="Post B Returns" sheetId="127" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="160">
   <si>
     <t>Total</t>
   </si>
@@ -419,6 +420,15 @@
     <t>Exit</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Max Series B per Share before Convert</t>
+  </si>
+  <si>
+    <t>Series B total Preferred Payment</t>
+  </si>
+  <si>
     <t>THINK MORE SECURITY &amp; 1011 VENTURES PRE-SERIES A</t>
   </si>
   <si>
@@ -489,6 +499,27 @@
   </si>
   <si>
     <t>MOIC for Series A Investment</t>
+  </si>
+  <si>
+    <t>Tier 1 Payments (SAFE, Series A &amp; B Preferred)</t>
+  </si>
+  <si>
+    <t>Aggregate Series B Preference at Point of Sale</t>
+  </si>
+  <si>
+    <t>Does Series B Convert/Lose Preference?</t>
+  </si>
+  <si>
+    <t>Series B Preferred Payment per Share</t>
+  </si>
+  <si>
+    <t>Other Common</t>
+  </si>
+  <si>
+    <t>ESOP/Pool</t>
+  </si>
+  <si>
+    <t>1011 Investment (Series A + Series B)</t>
   </si>
 </sst>
 </file>
@@ -1235,7 +1266,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1482,6 +1513,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="171" fontId="21" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="179" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -2955,7 +2989,7 @@
     <row r="4" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="32" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -2966,7 +3000,7 @@
     <row r="5" spans="1:7" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="32" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C5" s="32"/>
       <c r="D5" s="32"/>
@@ -3097,7 +3131,7 @@
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="34" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C13" s="9">
         <f>SUM('Detailed Cap Table'!D4:D20)+SUM('Detailed Cap Table'!E4:E20)</f>
@@ -3157,7 +3191,7 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="35" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="10"/>
@@ -3258,7 +3292,7 @@
     <row r="23" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C23" s="15">
         <f>D24/C25</f>
@@ -3285,7 +3319,7 @@
     <row r="25" spans="1:7" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C25" s="11">
         <f>F21</f>
@@ -3371,7 +3405,7 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="32" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C1" s="32"/>
       <c r="D1" s="32"/>
@@ -3390,7 +3424,7 @@
     <row r="2" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="32" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C2" s="32"/>
       <c r="D2" s="32"/>
@@ -3628,7 +3662,7 @@
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="34" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C11" s="9">
         <f>PreA!C13</f>
@@ -4026,7 +4060,7 @@
     <row r="25" spans="1:15" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="36" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C25" s="49"/>
       <c r="D25" s="49"/>
@@ -4152,7 +4186,7 @@
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C31" s="29">
         <v>0.1</v>
@@ -4195,7 +4229,7 @@
     <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C33" s="6">
         <f>I15</f>
@@ -4288,7 +4322,7 @@
     <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="32" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C1" s="32"/>
       <c r="D1" s="32"/>
@@ -4312,7 +4346,7 @@
     <row r="2" spans="1:20" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="32" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C2" s="32"/>
       <c r="D2" s="32"/>
@@ -4647,7 +4681,7 @@
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="34" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C11" s="71">
         <f>'Series A'!C11</f>
@@ -5449,7 +5483,7 @@
     <row r="33" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C33" s="29">
         <v>0.5</v>
@@ -5475,7 +5509,7 @@
     <row r="34" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C34" s="29">
         <v>7.0000000000000007E-2</v>
@@ -6181,7 +6215,7 @@
         <v>26</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -6801,7 +6835,7 @@
     <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -6845,7 +6879,7 @@
     <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -7247,7 +7281,7 @@
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" s="1"/>
       <c r="B49" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
@@ -7703,7 +7737,7 @@
     <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" s="1"/>
       <c r="B61" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -7765,7 +7799,7 @@
     <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" s="1"/>
       <c r="B63" s="17" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C63" s="95"/>
       <c r="D63" s="95"/>
@@ -7803,7 +7837,7 @@
     <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" s="1"/>
       <c r="B65" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
@@ -7847,7 +7881,7 @@
     <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" s="1"/>
       <c r="B66" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
@@ -7935,7 +7969,7 @@
     <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68" s="1"/>
       <c r="B68" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C68" s="1"/>
       <c r="D68" s="1"/>
@@ -7979,7 +8013,7 @@
     <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69" s="1"/>
       <c r="B69" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -8396,4 +8430,3266 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E7C45F5-ECA7-3A41-9716-F8F71000ED02}">
+  <dimension ref="A1:P100"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.1640625" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="6" width="11.1640625" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" customWidth="1"/>
+    <col min="8" max="8" width="11.1640625" customWidth="1"/>
+    <col min="9" max="16" width="17.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="88">
+        <f>I7/I5</f>
+        <v>25000000</v>
+      </c>
+      <c r="J4" s="88">
+        <f>J7/J5</f>
+        <v>33333333.333333332</v>
+      </c>
+      <c r="K4" s="88">
+        <f>K7/K5</f>
+        <v>41666666.666666664</v>
+      </c>
+      <c r="L4" s="88">
+        <f>L7/L5</f>
+        <v>50000000</v>
+      </c>
+      <c r="M4" s="88">
+        <f>M7/M5</f>
+        <v>58333333.333333336</v>
+      </c>
+      <c r="N4" s="88">
+        <f>N7/N5</f>
+        <v>66666666.666666664</v>
+      </c>
+      <c r="O4" s="88">
+        <f>O7/O5</f>
+        <v>83333333.333333328</v>
+      </c>
+      <c r="P4" s="88">
+        <f>P7/P5</f>
+        <v>125000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="98">
+        <v>6</v>
+      </c>
+      <c r="J5" s="98">
+        <v>6</v>
+      </c>
+      <c r="K5" s="98">
+        <v>6</v>
+      </c>
+      <c r="L5" s="98">
+        <v>6</v>
+      </c>
+      <c r="M5" s="98">
+        <v>6</v>
+      </c>
+      <c r="N5" s="98">
+        <v>6</v>
+      </c>
+      <c r="O5" s="98">
+        <v>6</v>
+      </c>
+      <c r="P5" s="98">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="56"/>
+      <c r="N6" s="56"/>
+      <c r="O6" s="56"/>
+      <c r="P6" s="56"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="87">
+        <v>150000000</v>
+      </c>
+      <c r="J7" s="87">
+        <v>200000000</v>
+      </c>
+      <c r="K7" s="87">
+        <v>250000000</v>
+      </c>
+      <c r="L7" s="87">
+        <v>300000000</v>
+      </c>
+      <c r="M7" s="87">
+        <v>350000000</v>
+      </c>
+      <c r="N7" s="87">
+        <v>400000000</v>
+      </c>
+      <c r="O7" s="87">
+        <v>500000000</v>
+      </c>
+      <c r="P7" s="87">
+        <v>750000000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="88"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="88"/>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="88"/>
+      <c r="O8" s="88"/>
+      <c r="P8" s="88"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A9" s="1"/>
+      <c r="B9" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="88"/>
+      <c r="L9" s="88"/>
+      <c r="M9" s="88"/>
+      <c r="N9" s="88"/>
+      <c r="O9" s="88"/>
+      <c r="P9" s="88"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="88"/>
+      <c r="L10" s="88"/>
+      <c r="M10" s="88"/>
+      <c r="N10" s="88"/>
+      <c r="O10" s="88"/>
+      <c r="P10" s="88"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="29">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="88">
+        <f>-$E$11*I7</f>
+        <v>-2250000</v>
+      </c>
+      <c r="J11" s="88">
+        <f>-$E$11*J7</f>
+        <v>-3000000</v>
+      </c>
+      <c r="K11" s="88">
+        <f>-$E$11*K7</f>
+        <v>-3750000</v>
+      </c>
+      <c r="L11" s="88">
+        <f>-$E$11*L7</f>
+        <v>-4500000</v>
+      </c>
+      <c r="M11" s="88">
+        <f>-$E$11*M7</f>
+        <v>-5250000</v>
+      </c>
+      <c r="N11" s="88">
+        <f>-$E$11*N7</f>
+        <v>-6000000</v>
+      </c>
+      <c r="O11" s="88">
+        <f>-$E$11*O7</f>
+        <v>-7500000</v>
+      </c>
+      <c r="P11" s="88">
+        <f>-$E$11*P7</f>
+        <v>-11250000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A12" s="1"/>
+      <c r="B12" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="94">
+        <f>I7+SUM(I8:I11)</f>
+        <v>147750000</v>
+      </c>
+      <c r="J12" s="94">
+        <f>J7+SUM(J8:J11)</f>
+        <v>197000000</v>
+      </c>
+      <c r="K12" s="94">
+        <f>K7+SUM(K8:K11)</f>
+        <v>246250000</v>
+      </c>
+      <c r="L12" s="94">
+        <f>L7+SUM(L8:L11)</f>
+        <v>295500000</v>
+      </c>
+      <c r="M12" s="94">
+        <f>M7+SUM(M8:M11)</f>
+        <v>344750000</v>
+      </c>
+      <c r="N12" s="94">
+        <f>N7+SUM(N8:N11)</f>
+        <v>394000000</v>
+      </c>
+      <c r="O12" s="94">
+        <f>O7+SUM(O8:O11)</f>
+        <v>492500000</v>
+      </c>
+      <c r="P12" s="94">
+        <f>P7+SUM(P8:P11)</f>
+        <v>738750000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="88"/>
+      <c r="J13" s="88"/>
+      <c r="K13" s="88"/>
+      <c r="L13" s="88"/>
+      <c r="M13" s="88"/>
+      <c r="N13" s="88"/>
+      <c r="O13" s="88"/>
+      <c r="P13" s="88"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="29">
+        <v>0.1</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="88">
+        <f ca="1">IF(I12&lt;(SUM(I19:I21)+($E$14*I12)),$E$14*I12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="88">
+        <f ca="1">IF(J12&lt;(SUM(J19:J21)+($E$14*J12)),$E$14*J12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="K14" s="88">
+        <f ca="1">IF(K12&lt;(SUM(K19:K21)+($E$14*K12)),$E$14*K12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L14" s="88">
+        <f ca="1">IF(L12&lt;(SUM(L19:L21)+($E$14*L12)),$E$14*L12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="M14" s="88">
+        <f ca="1">IF(M12&lt;(SUM(M19:M21)+($E$14*M12)),$E$14*M12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N14" s="88">
+        <f ca="1">IF(N12&lt;(SUM(N19:N21)+($E$14*N12)),$E$14*N12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O14" s="88">
+        <f ca="1">IF(O12&lt;(SUM(O19:O21)+($E$14*O12)),$E$14*O12,0)</f>
+        <v>0</v>
+      </c>
+      <c r="P14" s="88">
+        <f ca="1">IF(P12&lt;(SUM(P19:P21)+($E$14*P12)),$E$14*P12,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="88"/>
+      <c r="J15" s="88"/>
+      <c r="K15" s="88"/>
+      <c r="L15" s="88"/>
+      <c r="M15" s="88"/>
+      <c r="N15" s="88"/>
+      <c r="O15" s="88"/>
+      <c r="P15" s="88"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" s="1"/>
+      <c r="B16" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="89">
+        <f ca="1">I12-I14</f>
+        <v>147750000</v>
+      </c>
+      <c r="J16" s="89">
+        <f ca="1">J12-J14</f>
+        <v>197000000</v>
+      </c>
+      <c r="K16" s="89">
+        <f ca="1">K12-K14</f>
+        <v>246250000</v>
+      </c>
+      <c r="L16" s="89">
+        <f ca="1">L12-L14</f>
+        <v>295500000</v>
+      </c>
+      <c r="M16" s="89">
+        <f ca="1">M12-M14</f>
+        <v>344750000</v>
+      </c>
+      <c r="N16" s="89">
+        <f ca="1">N12-N14</f>
+        <v>394000000</v>
+      </c>
+      <c r="O16" s="89">
+        <f ca="1">O12-O14</f>
+        <v>492500000</v>
+      </c>
+      <c r="P16" s="89">
+        <f ca="1">P12-P14</f>
+        <v>738750000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="56"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="56"/>
+      <c r="O17" s="56"/>
+      <c r="P17" s="56"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I18" s="56"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="56"/>
+      <c r="M18" s="56"/>
+      <c r="N18" s="56"/>
+      <c r="O18" s="56"/>
+      <c r="P18" s="56"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+      <c r="F19" s="8">
+        <f>'Series A'!E22</f>
+        <v>4.1246319529565065</v>
+      </c>
+      <c r="G19" s="5">
+        <f>'Series A'!E21</f>
+        <v>2382031</v>
+      </c>
+      <c r="H19" s="7">
+        <f ca="1">I19/SUM($I$19:$I$21)</f>
+        <v>0.16422900033775137</v>
+      </c>
+      <c r="I19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="J19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="K19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="L19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="M19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="N19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="O19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="P19" s="88">
+        <f>$G19*$F19*$E19</f>
+        <v>9825001.1755329408</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1">
+        <v>1</v>
+      </c>
+      <c r="F20" s="8">
+        <f ca="1">'Series A'!J22</f>
+        <v>4.3128000000000002</v>
+      </c>
+      <c r="G20" s="5">
+        <f ca="1">'Series A'!J21</f>
+        <v>4637359</v>
+      </c>
+      <c r="H20" s="7">
+        <f ca="1">I20/SUM($I$19:$I$21)</f>
+        <v>0.33430838931412771</v>
+      </c>
+      <c r="I20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="J20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="K20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="L20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="M20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="N20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="O20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="P20" s="88">
+        <f ca="1">$G20*$F20*$E20</f>
+        <v>20000001.895199999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+      <c r="F21" s="8">
+        <f ca="1">'Series B'!O24</f>
+        <v>7.4071999999999996</v>
+      </c>
+      <c r="G21" s="5">
+        <f ca="1">'Series B'!O22</f>
+        <v>4050114</v>
+      </c>
+      <c r="H21" s="7">
+        <f ca="1">I21/SUM($I$19:$I$21)</f>
+        <v>0.5014626103481209</v>
+      </c>
+      <c r="I21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="J21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="K21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="L21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="M21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="N21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="O21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="P21" s="88">
+        <f ca="1">$G21*$F21*$E21</f>
+        <v>30000004.420799997</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="56"/>
+      <c r="J22" s="56"/>
+      <c r="K22" s="56"/>
+      <c r="L22" s="56"/>
+      <c r="M22" s="56"/>
+      <c r="N22" s="56"/>
+      <c r="O22" s="56"/>
+      <c r="P22" s="56"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="56"/>
+      <c r="K23" s="56"/>
+      <c r="L23" s="56"/>
+      <c r="M23" s="56"/>
+      <c r="N23" s="56"/>
+      <c r="O23" s="56"/>
+      <c r="P23" s="56"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="56"/>
+      <c r="M24" s="56"/>
+      <c r="N24" s="56"/>
+      <c r="O24" s="56"/>
+      <c r="P24" s="56"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="88">
+        <f>I19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="J25" s="88">
+        <f>J19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="K25" s="88">
+        <f>K19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="L25" s="88">
+        <f>L19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="M25" s="88">
+        <f>M19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="N25" s="88">
+        <f>N19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="O25" s="88">
+        <f>O19</f>
+        <v>9825001.1755329408</v>
+      </c>
+      <c r="P25" s="88">
+        <f>P19</f>
+        <v>9825001.1755329408</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;I$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="J26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;J$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="K26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;K$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="L26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;L$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="M26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;M$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="N26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;N$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="O26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;O$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="P26" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$19&lt;P$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="88">
+        <f ca="1">IF(I14=0,IF(I26="yes",0,I$19),$H$19*I16)</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="88">
+        <f ca="1">IF(J14=0,IF(J26="yes",0,J$19),$H$19*J16)</f>
+        <v>0</v>
+      </c>
+      <c r="K27" s="88">
+        <f ca="1">IF(K14=0,IF(K26="yes",0,K$19),$H$19*K16)</f>
+        <v>0</v>
+      </c>
+      <c r="L27" s="88">
+        <f ca="1">IF(L14=0,IF(L26="yes",0,L$19),$H$19*L16)</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="88">
+        <f ca="1">IF(M14=0,IF(M26="yes",0,M$19),$H$19*M16)</f>
+        <v>0</v>
+      </c>
+      <c r="N27" s="88">
+        <f ca="1">IF(N14=0,IF(N26="yes",0,N$19),$H$19*N16)</f>
+        <v>0</v>
+      </c>
+      <c r="O27" s="88">
+        <f ca="1">IF(O14=0,IF(O26="yes",0,O$19),$H$19*O16)</f>
+        <v>0</v>
+      </c>
+      <c r="P27" s="88">
+        <f ca="1">IF(P14=0,IF(P26="yes",0,P$19),$H$19*P16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="88">
+        <f ca="1">I27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="88">
+        <f ca="1">J27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="K28" s="88">
+        <f ca="1">K27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="L28" s="88">
+        <f ca="1">L27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="M28" s="88">
+        <f ca="1">M27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="N28" s="88">
+        <f ca="1">N27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="O28" s="88">
+        <f ca="1">O27/$G$19</f>
+        <v>0</v>
+      </c>
+      <c r="P28" s="88">
+        <f ca="1">P27/$G$19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="88"/>
+      <c r="J29" s="88"/>
+      <c r="K29" s="88"/>
+      <c r="L29" s="88"/>
+      <c r="M29" s="88"/>
+      <c r="N29" s="88"/>
+      <c r="O29" s="88"/>
+      <c r="P29" s="88"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="88">
+        <f ca="1">I20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="J30" s="88">
+        <f ca="1">J20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="K30" s="88">
+        <f ca="1">K20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="L30" s="88">
+        <f ca="1">L20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="M30" s="88">
+        <f ca="1">M20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="N30" s="88">
+        <f ca="1">N20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="O30" s="88">
+        <f ca="1">O20</f>
+        <v>20000001.895199999</v>
+      </c>
+      <c r="P30" s="88">
+        <f ca="1">P20</f>
+        <v>20000001.895199999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;I$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="J31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;J$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="K31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;K$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="L31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;L$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="M31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;M$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="N31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;N$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="O31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;O$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="P31" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$20&lt;P$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="88">
+        <f ca="1">IF(I14=0,IF(I31="yes",0,I$20),$H$20*I16)</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="88">
+        <f ca="1">IF(J14=0,IF(J31="yes",0,J$20),$H$20*J16)</f>
+        <v>0</v>
+      </c>
+      <c r="K32" s="88">
+        <f ca="1">IF(K14=0,IF(K31="yes",0,K$20),$H$20*K16)</f>
+        <v>0</v>
+      </c>
+      <c r="L32" s="88">
+        <f ca="1">IF(L14=0,IF(L31="yes",0,L$20),$H$20*L16)</f>
+        <v>0</v>
+      </c>
+      <c r="M32" s="88">
+        <f ca="1">IF(M14=0,IF(M31="yes",0,M$20),$H$20*M16)</f>
+        <v>0</v>
+      </c>
+      <c r="N32" s="88">
+        <f ca="1">IF(N14=0,IF(N31="yes",0,N$20),$H$20*N16)</f>
+        <v>0</v>
+      </c>
+      <c r="O32" s="88">
+        <f ca="1">IF(O14=0,IF(O31="yes",0,O$20),$H$20*O16)</f>
+        <v>0</v>
+      </c>
+      <c r="P32" s="88">
+        <f ca="1">IF(P14=0,IF(P31="yes",0,P$20),$H$20*P16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="88">
+        <f ca="1">I32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="88">
+        <f ca="1">J32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="K33" s="88">
+        <f ca="1">K32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="L33" s="88">
+        <f ca="1">L32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="M33" s="88">
+        <f ca="1">M32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="N33" s="88">
+        <f ca="1">N32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="O33" s="88">
+        <f ca="1">O32/$G$20</f>
+        <v>0</v>
+      </c>
+      <c r="P33" s="88">
+        <f ca="1">P32/$G$20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="I34" s="88"/>
+      <c r="J34" s="88"/>
+      <c r="K34" s="88"/>
+      <c r="L34" s="88"/>
+      <c r="M34" s="88"/>
+      <c r="N34" s="88"/>
+      <c r="O34" s="88"/>
+      <c r="P34" s="88"/>
+    </row>
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="88">
+        <f ca="1">I21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="J35" s="88">
+        <f ca="1">J21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="K35" s="88">
+        <f ca="1">K21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="L35" s="88">
+        <f ca="1">L21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="M35" s="88">
+        <f ca="1">M21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="N35" s="88">
+        <f ca="1">N21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="O35" s="88">
+        <f ca="1">O21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="P35" s="88">
+        <f ca="1">P21</f>
+        <v>30000004.420799997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
+      <c r="I36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;I$44,"yes","no"),0)</f>
+        <v>no</v>
+      </c>
+      <c r="J36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;J$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="K36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;K$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="L36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;L$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="M36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;M$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="N36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;N$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="O36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;O$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+      <c r="P36" s="88" t="str">
+        <f ca="1">IFERROR(IF($F$21&lt;P$44,"yes","no"),0)</f>
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="88">
+        <f ca="1">IF(I14=0,IF(I36="yes",0,I$21),$H$21*I16)</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="J37" s="88">
+        <f ca="1">IF(J14=0,IF(J36="yes",0,J$21),$H$21*J16)</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="88">
+        <f ca="1">IF(K14=0,IF(K36="yes",0,K$21),$H$21*K16)</f>
+        <v>0</v>
+      </c>
+      <c r="L37" s="88">
+        <f ca="1">IF(L14=0,IF(L36="yes",0,L$21),$H$21*L16)</f>
+        <v>0</v>
+      </c>
+      <c r="M37" s="88">
+        <f ca="1">IF(M14=0,IF(M36="yes",0,M$21),$H$21*M16)</f>
+        <v>0</v>
+      </c>
+      <c r="N37" s="88">
+        <f ca="1">IF(N14=0,IF(N36="yes",0,N$21),$H$21*N16)</f>
+        <v>0</v>
+      </c>
+      <c r="O37" s="88">
+        <f ca="1">IF(O14=0,IF(O36="yes",0,O$21),$H$21*O16)</f>
+        <v>0</v>
+      </c>
+      <c r="P37" s="88">
+        <f ca="1">IF(P14=0,IF(P36="yes",0,P$21),$H$21*P16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="88">
+        <f ca="1">I37/$G$21</f>
+        <v>7.4071999999999996</v>
+      </c>
+      <c r="J38" s="88">
+        <f ca="1">J37/$G$21</f>
+        <v>0</v>
+      </c>
+      <c r="K38" s="88">
+        <f ca="1">K37/$G$21</f>
+        <v>0</v>
+      </c>
+      <c r="L38" s="88">
+        <f ca="1">L37/$G$21</f>
+        <v>0</v>
+      </c>
+      <c r="M38" s="88">
+        <f ca="1">M37/$G$21</f>
+        <v>0</v>
+      </c>
+      <c r="N38" s="88">
+        <f ca="1">N37/$G$21</f>
+        <v>0</v>
+      </c>
+      <c r="O38" s="88">
+        <f ca="1">O37/$G$21</f>
+        <v>0</v>
+      </c>
+      <c r="P38" s="88">
+        <f ca="1">P37/$G$21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1"/>
+      <c r="I39" s="88"/>
+      <c r="J39" s="88"/>
+      <c r="K39" s="88"/>
+      <c r="L39" s="88"/>
+      <c r="M39" s="88"/>
+      <c r="N39" s="88"/>
+      <c r="O39" s="88"/>
+      <c r="P39" s="88"/>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1"/>
+      <c r="I40" s="88">
+        <f ca="1">I16-I27-I32-I37</f>
+        <v>117749995.5792</v>
+      </c>
+      <c r="J40" s="88">
+        <f ca="1">J16-J27-J32-J37</f>
+        <v>197000000</v>
+      </c>
+      <c r="K40" s="88">
+        <f ca="1">K16-K27-K32-K37</f>
+        <v>246250000</v>
+      </c>
+      <c r="L40" s="88">
+        <f ca="1">L16-L27-L32-L37</f>
+        <v>295500000</v>
+      </c>
+      <c r="M40" s="88">
+        <f ca="1">M16-M27-M32-M37</f>
+        <v>344750000</v>
+      </c>
+      <c r="N40" s="88">
+        <f ca="1">N16-N27-N32-N37</f>
+        <v>394000000</v>
+      </c>
+      <c r="O40" s="88">
+        <f ca="1">O16-O27-O32-O37</f>
+        <v>492500000</v>
+      </c>
+      <c r="P40" s="88">
+        <f ca="1">P16-P27-P32-P37</f>
+        <v>738750000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1"/>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="56"/>
+      <c r="K41" s="56"/>
+      <c r="L41" s="56"/>
+      <c r="M41" s="56"/>
+      <c r="N41" s="56"/>
+      <c r="O41" s="56"/>
+      <c r="P41" s="56"/>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A42" s="1"/>
+      <c r="B42" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1"/>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="56"/>
+      <c r="K42" s="56"/>
+      <c r="L42" s="56"/>
+      <c r="M42" s="56"/>
+      <c r="N42" s="56"/>
+      <c r="O42" s="56"/>
+      <c r="P42" s="56"/>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1"/>
+      <c r="I43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(I26="yes",$G$19,0)+IF(I31="yes",$G$20,0)+IF(I36="yes",$G$21,0)</f>
+        <v>20250544</v>
+      </c>
+      <c r="J43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(J26="yes",$G$19,0)+IF(J31="yes",$G$20,0)+IF(J36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+      <c r="K43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(K26="yes",$G$19,0)+IF(K31="yes",$G$20,0)+IF(K36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+      <c r="L43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(L26="yes",$G$19,0)+IF(L31="yes",$G$20,0)+IF(L36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+      <c r="M43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(M26="yes",$G$19,0)+IF(M31="yes",$G$20,0)+IF(M36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+      <c r="N43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(N26="yes",$G$19,0)+IF(N31="yes",$G$20,0)+IF(N36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+      <c r="O43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(O26="yes",$G$19,0)+IF(O31="yes",$G$20,0)+IF(O36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+      <c r="P43" s="90">
+        <f ca="1">'Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12+IF(P26="yes",$G$19,0)+IF(P31="yes",$G$20,0)+IF(P36="yes",$G$21,0)</f>
+        <v>24300658</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1"/>
+      <c r="I44" s="90">
+        <f ca="1">IFERROR(I40/I43,0)</f>
+        <v>5.8146583903721298</v>
+      </c>
+      <c r="J44" s="90">
+        <f ca="1">IFERROR(J40/J43,0)</f>
+        <v>8.1067763679485552</v>
+      </c>
+      <c r="K44" s="90">
+        <f ca="1">IFERROR(K40/K43,0)</f>
+        <v>10.133470459935694</v>
+      </c>
+      <c r="L44" s="90">
+        <f ca="1">IFERROR(L40/L43,0)</f>
+        <v>12.160164551922833</v>
+      </c>
+      <c r="M44" s="90">
+        <f ca="1">IFERROR(M40/M43,0)</f>
+        <v>14.186858643909972</v>
+      </c>
+      <c r="N44" s="90">
+        <f ca="1">IFERROR(N40/N43,0)</f>
+        <v>16.21355273589711</v>
+      </c>
+      <c r="O44" s="90">
+        <f ca="1">IFERROR(O40/O43,0)</f>
+        <v>20.266940919871388</v>
+      </c>
+      <c r="P44" s="90">
+        <f ca="1">IFERROR(P40/P43,0)</f>
+        <v>30.400411379807082</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="56"/>
+      <c r="J45" s="56"/>
+      <c r="K45" s="56"/>
+      <c r="L45" s="56"/>
+      <c r="M45" s="56"/>
+      <c r="N45" s="56"/>
+      <c r="O45" s="56"/>
+      <c r="P45" s="56"/>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A46" s="1"/>
+      <c r="B46" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1"/>
+      <c r="I46" s="56"/>
+      <c r="J46" s="56"/>
+      <c r="K46" s="56"/>
+      <c r="L46" s="56"/>
+      <c r="M46" s="56"/>
+      <c r="N46" s="56"/>
+      <c r="O46" s="56"/>
+      <c r="P46" s="56"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
+      <c r="I47" s="91">
+        <f ca="1">IF(I26="yes",I44,I28)</f>
+        <v>5.8146583903721298</v>
+      </c>
+      <c r="J47" s="91">
+        <f ca="1">IF(J26="yes",J44,J28)</f>
+        <v>8.1067763679485552</v>
+      </c>
+      <c r="K47" s="91">
+        <f ca="1">IF(K26="yes",K44,K28)</f>
+        <v>10.133470459935694</v>
+      </c>
+      <c r="L47" s="91">
+        <f ca="1">IF(L26="yes",L44,L28)</f>
+        <v>12.160164551922833</v>
+      </c>
+      <c r="M47" s="91">
+        <f ca="1">IF(M26="yes",M44,M28)</f>
+        <v>14.186858643909972</v>
+      </c>
+      <c r="N47" s="91">
+        <f ca="1">IF(N26="yes",N44,N28)</f>
+        <v>16.21355273589711</v>
+      </c>
+      <c r="O47" s="91">
+        <f ca="1">IF(O26="yes",O44,O28)</f>
+        <v>20.266940919871388</v>
+      </c>
+      <c r="P47" s="91">
+        <f ca="1">IF(P26="yes",P44,P28)</f>
+        <v>30.400411379807082</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
+      <c r="I48" s="91">
+        <f ca="1">IF(I31="yes",I44,I33)</f>
+        <v>5.8146583903721298</v>
+      </c>
+      <c r="J48" s="91">
+        <f ca="1">IF(J31="yes",J44,J33)</f>
+        <v>8.1067763679485552</v>
+      </c>
+      <c r="K48" s="91">
+        <f ca="1">IF(K31="yes",K44,K33)</f>
+        <v>10.133470459935694</v>
+      </c>
+      <c r="L48" s="91">
+        <f ca="1">IF(L31="yes",L44,L33)</f>
+        <v>12.160164551922833</v>
+      </c>
+      <c r="M48" s="91">
+        <f ca="1">IF(M31="yes",M44,M33)</f>
+        <v>14.186858643909972</v>
+      </c>
+      <c r="N48" s="91">
+        <f ca="1">IF(N31="yes",N44,N33)</f>
+        <v>16.21355273589711</v>
+      </c>
+      <c r="O48" s="91">
+        <f ca="1">IF(O31="yes",O44,O33)</f>
+        <v>20.266940919871388</v>
+      </c>
+      <c r="P48" s="91">
+        <f ca="1">IF(P31="yes",P44,P33)</f>
+        <v>30.400411379807082</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1"/>
+      <c r="H49" s="1"/>
+      <c r="I49" s="91">
+        <f ca="1">IF(I36="yes",I44,I38)</f>
+        <v>7.4071999999999996</v>
+      </c>
+      <c r="J49" s="91">
+        <f ca="1">IF(J36="yes",J44,J38)</f>
+        <v>8.1067763679485552</v>
+      </c>
+      <c r="K49" s="91">
+        <f ca="1">IF(K36="yes",K44,K38)</f>
+        <v>10.133470459935694</v>
+      </c>
+      <c r="L49" s="91">
+        <f ca="1">IF(L36="yes",L44,L38)</f>
+        <v>12.160164551922833</v>
+      </c>
+      <c r="M49" s="91">
+        <f ca="1">IF(M36="yes",M44,M38)</f>
+        <v>14.186858643909972</v>
+      </c>
+      <c r="N49" s="91">
+        <f ca="1">IF(N36="yes",N44,N38)</f>
+        <v>16.21355273589711</v>
+      </c>
+      <c r="O49" s="91">
+        <f ca="1">IF(O36="yes",O44,O38)</f>
+        <v>20.266940919871388</v>
+      </c>
+      <c r="P49" s="91">
+        <f ca="1">IF(P36="yes",P44,P38)</f>
+        <v>30.400411379807082</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A50" s="1"/>
+      <c r="B50" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1"/>
+      <c r="H50" s="1"/>
+      <c r="I50" s="91">
+        <f ca="1">I44</f>
+        <v>5.8146583903721298</v>
+      </c>
+      <c r="J50" s="91">
+        <f ca="1">J44</f>
+        <v>8.1067763679485552</v>
+      </c>
+      <c r="K50" s="91">
+        <f ca="1">K44</f>
+        <v>10.133470459935694</v>
+      </c>
+      <c r="L50" s="91">
+        <f ca="1">L44</f>
+        <v>12.160164551922833</v>
+      </c>
+      <c r="M50" s="91">
+        <f ca="1">M44</f>
+        <v>14.186858643909972</v>
+      </c>
+      <c r="N50" s="91">
+        <f ca="1">N44</f>
+        <v>16.21355273589711</v>
+      </c>
+      <c r="O50" s="91">
+        <f ca="1">O44</f>
+        <v>20.266940919871388</v>
+      </c>
+      <c r="P50" s="91">
+        <f ca="1">P44</f>
+        <v>30.400411379807082</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="1"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1"/>
+      <c r="H51" s="1"/>
+      <c r="I51" s="56"/>
+      <c r="J51" s="56"/>
+      <c r="K51" s="56"/>
+      <c r="L51" s="56"/>
+      <c r="M51" s="56"/>
+      <c r="N51" s="56"/>
+      <c r="O51" s="56"/>
+      <c r="P51" s="56"/>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A52" s="1"/>
+      <c r="B52" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C52" s="1"/>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1"/>
+      <c r="H52" s="1"/>
+      <c r="I52" s="56"/>
+      <c r="J52" s="56"/>
+      <c r="K52" s="56"/>
+      <c r="L52" s="56"/>
+      <c r="M52" s="56"/>
+      <c r="N52" s="56"/>
+      <c r="O52" s="56"/>
+      <c r="P52" s="56"/>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
+      <c r="I53" s="88">
+        <f ca="1">I47*$G$19</f>
+        <v>13850696.540276514</v>
+      </c>
+      <c r="J53" s="88">
+        <f ca="1">J47*$G$19</f>
+        <v>19310592.618520863</v>
+      </c>
+      <c r="K53" s="88">
+        <f ca="1">K47*$G$19</f>
+        <v>24138240.773151081</v>
+      </c>
+      <c r="L53" s="88">
+        <f ca="1">L47*$G$19</f>
+        <v>28965888.927781299</v>
+      </c>
+      <c r="M53" s="88">
+        <f ca="1">M47*$G$19</f>
+        <v>33793537.082411513</v>
+      </c>
+      <c r="N53" s="88">
+        <f ca="1">N47*$G$19</f>
+        <v>38621185.237041727</v>
+      </c>
+      <c r="O53" s="88">
+        <f ca="1">O47*$G$19</f>
+        <v>48276481.546302162</v>
+      </c>
+      <c r="P53" s="88">
+        <f ca="1">P47*$G$19</f>
+        <v>72414722.319453239</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A54" s="1"/>
+      <c r="B54" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
+      <c r="I54" s="88">
+        <f ca="1">I48*$G$20</f>
+        <v>26964658.418517709</v>
+      </c>
+      <c r="J54" s="88">
+        <f ca="1">J48*$G$20</f>
+        <v>37594032.350893542</v>
+      </c>
+      <c r="K54" s="88">
+        <f ca="1">K48*$G$20</f>
+        <v>46992540.438616931</v>
+      </c>
+      <c r="L54" s="88">
+        <f ca="1">L48*$G$20</f>
+        <v>56391048.526340313</v>
+      </c>
+      <c r="M54" s="88">
+        <f ca="1">M48*$G$20</f>
+        <v>65789556.614063703</v>
+      </c>
+      <c r="N54" s="88">
+        <f ca="1">N48*$G$20</f>
+        <v>75188064.701787084</v>
+      </c>
+      <c r="O54" s="88">
+        <f ca="1">O48*$G$20</f>
+        <v>93985080.877233863</v>
+      </c>
+      <c r="P54" s="88">
+        <f ca="1">P48*$G$20</f>
+        <v>140977621.31585079</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A55" s="1"/>
+      <c r="B55" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="88">
+        <f ca="1">I49*$G$21</f>
+        <v>30000004.420799997</v>
+      </c>
+      <c r="J55" s="88">
+        <f ca="1">J49*$G$21</f>
+        <v>32833368.462697595</v>
+      </c>
+      <c r="K55" s="88">
+        <f ca="1">K49*$G$21</f>
+        <v>41041710.578371994</v>
+      </c>
+      <c r="L55" s="88">
+        <f ca="1">L49*$G$21</f>
+        <v>49250052.694046393</v>
+      </c>
+      <c r="M55" s="88">
+        <f ca="1">M49*$G$21</f>
+        <v>57458394.809720792</v>
+      </c>
+      <c r="N55" s="88">
+        <f ca="1">N49*$G$21</f>
+        <v>65666736.925395191</v>
+      </c>
+      <c r="O55" s="88">
+        <f ca="1">O49*$G$21</f>
+        <v>82083421.156743988</v>
+      </c>
+      <c r="P55" s="88">
+        <f ca="1">P49*$G$21</f>
+        <v>123125131.73511598</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A56" s="1"/>
+      <c r="B56" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
+      <c r="I56" s="88">
+        <f ca="1">I50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>76934640.620405763</v>
+      </c>
+      <c r="J56" s="88">
+        <f ca="1">J50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>107262006.56788799</v>
+      </c>
+      <c r="K56" s="88">
+        <f ca="1">K50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>134077508.20986</v>
+      </c>
+      <c r="L56" s="88">
+        <f ca="1">L50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>160893009.851832</v>
+      </c>
+      <c r="M56" s="88">
+        <f ca="1">M50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>187708511.49380401</v>
+      </c>
+      <c r="N56" s="88">
+        <f ca="1">N50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>214524013.13577598</v>
+      </c>
+      <c r="O56" s="88">
+        <f ca="1">O50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>268155016.41971999</v>
+      </c>
+      <c r="P56" s="88">
+        <f ca="1">P50*('Series A'!$C$13+'Series A'!$L$12+'Series B'!$Q$12)</f>
+        <v>402232524.62957996</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A57" s="1"/>
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
+      <c r="I57" s="88"/>
+      <c r="J57" s="88"/>
+      <c r="K57" s="88"/>
+      <c r="L57" s="88"/>
+      <c r="M57" s="88"/>
+      <c r="N57" s="88"/>
+      <c r="O57" s="88"/>
+      <c r="P57" s="88"/>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A58" s="1"/>
+      <c r="B58" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
+      <c r="I58" s="88">
+        <f ca="1">SUM(I53:I56)-I16</f>
+        <v>0</v>
+      </c>
+      <c r="J58" s="88">
+        <f ca="1">SUM(J53:J56)-J16</f>
+        <v>0</v>
+      </c>
+      <c r="K58" s="88">
+        <f ca="1">SUM(K53:K56)-K16</f>
+        <v>0</v>
+      </c>
+      <c r="L58" s="88">
+        <f ca="1">SUM(L53:L56)-L16</f>
+        <v>0</v>
+      </c>
+      <c r="M58" s="88">
+        <f ca="1">SUM(M53:M56)-M16</f>
+        <v>0</v>
+      </c>
+      <c r="N58" s="88">
+        <f ca="1">SUM(N53:N56)-N16</f>
+        <v>0</v>
+      </c>
+      <c r="O58" s="88">
+        <f ca="1">SUM(O53:O56)-O16</f>
+        <v>0</v>
+      </c>
+      <c r="P58" s="88">
+        <f ca="1">SUM(P53:P56)-P16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A59" s="1"/>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="56"/>
+      <c r="J59" s="56"/>
+      <c r="K59" s="56"/>
+      <c r="L59" s="56"/>
+      <c r="M59" s="56"/>
+      <c r="N59" s="56"/>
+      <c r="O59" s="56"/>
+      <c r="P59" s="56"/>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A60" s="1"/>
+      <c r="B60" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="56"/>
+      <c r="J60" s="56"/>
+      <c r="K60" s="56"/>
+      <c r="L60" s="56"/>
+      <c r="M60" s="56"/>
+      <c r="N60" s="56"/>
+      <c r="O60" s="56"/>
+      <c r="P60" s="56"/>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
+      <c r="I61" s="88">
+        <f ca="1">I$47*'Series B'!$E8+I$48*'Series B'!$J8+I$49*'Series B'!$O8+I$50*'Series B'!$C8</f>
+        <v>20932770.205339666</v>
+      </c>
+      <c r="J61" s="88">
+        <f ca="1">J$47*'Series B'!$E8+J$48*'Series B'!$J8+J$49*'Series B'!$O8+J$50*'Series B'!$C8</f>
+        <v>29184394.924614798</v>
+      </c>
+      <c r="K61" s="88">
+        <f ca="1">K$47*'Series B'!$E8+K$48*'Series B'!$J8+K$49*'Series B'!$O8+K$50*'Series B'!$C8</f>
+        <v>36480493.655768499</v>
+      </c>
+      <c r="L61" s="88">
+        <f ca="1">L$47*'Series B'!$E8+L$48*'Series B'!$J8+L$49*'Series B'!$O8+L$50*'Series B'!$C8</f>
+        <v>43776592.386922196</v>
+      </c>
+      <c r="M61" s="88">
+        <f ca="1">M$47*'Series B'!$E8+M$48*'Series B'!$J8+M$49*'Series B'!$O8+M$50*'Series B'!$C8</f>
+        <v>51072691.1180759</v>
+      </c>
+      <c r="N61" s="88">
+        <f ca="1">N$47*'Series B'!$E8+N$48*'Series B'!$J8+N$49*'Series B'!$O8+N$50*'Series B'!$C8</f>
+        <v>58368789.849229597</v>
+      </c>
+      <c r="O61" s="88">
+        <f ca="1">O$47*'Series B'!$E8+O$48*'Series B'!$J8+O$49*'Series B'!$O8+O$50*'Series B'!$C8</f>
+        <v>72960987.311536998</v>
+      </c>
+      <c r="P61" s="88">
+        <f ca="1">P$47*'Series B'!$E8+P$48*'Series B'!$J8+P$49*'Series B'!$O8+P$50*'Series B'!$C8</f>
+        <v>109441480.9673055</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" s="1"/>
+      <c r="D62" s="1"/>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1"/>
+      <c r="G62" s="1"/>
+      <c r="H62" s="1"/>
+      <c r="I62" s="88">
+        <f ca="1">I$47*'Series B'!$E9+I$48*'Series B'!$J9+I$49*'Series B'!$O9+I$50*'Series B'!$C9</f>
+        <v>20932770.205339666</v>
+      </c>
+      <c r="J62" s="88">
+        <f ca="1">J$47*'Series B'!$E9+J$48*'Series B'!$J9+J$49*'Series B'!$O9+J$50*'Series B'!$C9</f>
+        <v>29184394.924614798</v>
+      </c>
+      <c r="K62" s="88">
+        <f ca="1">K$47*'Series B'!$E9+K$48*'Series B'!$J9+K$49*'Series B'!$O9+K$50*'Series B'!$C9</f>
+        <v>36480493.655768499</v>
+      </c>
+      <c r="L62" s="88">
+        <f ca="1">L$47*'Series B'!$E9+L$48*'Series B'!$J9+L$49*'Series B'!$O9+L$50*'Series B'!$C9</f>
+        <v>43776592.386922196</v>
+      </c>
+      <c r="M62" s="88">
+        <f ca="1">M$47*'Series B'!$E9+M$48*'Series B'!$J9+M$49*'Series B'!$O9+M$50*'Series B'!$C9</f>
+        <v>51072691.1180759</v>
+      </c>
+      <c r="N62" s="88">
+        <f ca="1">N$47*'Series B'!$E9+N$48*'Series B'!$J9+N$49*'Series B'!$O9+N$50*'Series B'!$C9</f>
+        <v>58368789.849229597</v>
+      </c>
+      <c r="O62" s="88">
+        <f ca="1">O$47*'Series B'!$E9+O$48*'Series B'!$J9+O$49*'Series B'!$O9+O$50*'Series B'!$C9</f>
+        <v>72960987.311536998</v>
+      </c>
+      <c r="P62" s="88">
+        <f ca="1">P$47*'Series B'!$E9+P$48*'Series B'!$J9+P$49*'Series B'!$O9+P$50*'Series B'!$C9</f>
+        <v>109441480.9673055</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C63" s="1"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="88">
+        <f ca="1">I$47*'Series B'!$E10+I$48*'Series B'!$J10+I$49*'Series B'!$O10+I$50*'Series B'!$C10</f>
+        <v>8433667.7492715921</v>
+      </c>
+      <c r="J63" s="88">
+        <f ca="1">J$47*'Series B'!$E10+J$48*'Series B'!$J10+J$49*'Series B'!$O10+J$50*'Series B'!$C10</f>
+        <v>11758190.045718104</v>
+      </c>
+      <c r="K63" s="88">
+        <f ca="1">K$47*'Series B'!$E10+K$48*'Series B'!$J10+K$49*'Series B'!$O10+K$50*'Series B'!$C10</f>
+        <v>14697737.55714763</v>
+      </c>
+      <c r="L63" s="88">
+        <f ca="1">L$47*'Series B'!$E10+L$48*'Series B'!$J10+L$49*'Series B'!$O10+L$50*'Series B'!$C10</f>
+        <v>17637285.068577155</v>
+      </c>
+      <c r="M63" s="88">
+        <f ca="1">M$47*'Series B'!$E10+M$48*'Series B'!$J10+M$49*'Series B'!$O10+M$50*'Series B'!$C10</f>
+        <v>20576832.580006681</v>
+      </c>
+      <c r="N63" s="88">
+        <f ca="1">N$47*'Series B'!$E10+N$48*'Series B'!$J10+N$49*'Series B'!$O10+N$50*'Series B'!$C10</f>
+        <v>23516380.091436207</v>
+      </c>
+      <c r="O63" s="88">
+        <f ca="1">O$47*'Series B'!$E10+O$48*'Series B'!$J10+O$49*'Series B'!$O10+O$50*'Series B'!$C10</f>
+        <v>29395475.114295259</v>
+      </c>
+      <c r="P63" s="88">
+        <f ca="1">P$47*'Series B'!$E10+P$48*'Series B'!$J10+P$49*'Series B'!$O10+P$50*'Series B'!$C10</f>
+        <v>44093212.671442889</v>
+      </c>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A64" s="1"/>
+      <c r="B64" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C64" s="1"/>
+      <c r="D64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1"/>
+      <c r="G64" s="1"/>
+      <c r="H64" s="1"/>
+      <c r="I64" s="88">
+        <f ca="1">I$47*'Series B'!$E11+I$48*'Series B'!$J11+I$49*'Series B'!$O11+I$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>26635432.46045484</v>
+      </c>
+      <c r="J64" s="88">
+        <f ca="1">J$47*'Series B'!$E11+J$48*'Series B'!$J11+J$49*'Series B'!$O11+J$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>37135026.672940299</v>
+      </c>
+      <c r="K64" s="88">
+        <f ca="1">K$47*'Series B'!$E11+K$48*'Series B'!$J11+K$49*'Series B'!$O11+K$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>46418783.34117537</v>
+      </c>
+      <c r="L64" s="88">
+        <f ca="1">L$47*'Series B'!$E11+L$48*'Series B'!$J11+L$49*'Series B'!$O11+L$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>55702540.009410448</v>
+      </c>
+      <c r="M64" s="88">
+        <f ca="1">M$47*'Series B'!$E11+M$48*'Series B'!$J11+M$49*'Series B'!$O11+M$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>64986296.677645519</v>
+      </c>
+      <c r="N64" s="88">
+        <f ca="1">N$47*'Series B'!$E11+N$48*'Series B'!$J11+N$49*'Series B'!$O11+N$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>74270053.345880598</v>
+      </c>
+      <c r="O64" s="88">
+        <f ca="1">O$47*'Series B'!$E11+O$48*'Series B'!$J11+O$49*'Series B'!$O11+O$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>92837566.68235074</v>
+      </c>
+      <c r="P64" s="88">
+        <f ca="1">P$47*'Series B'!$E11+P$48*'Series B'!$J11+P$49*'Series B'!$O11+P$50*('Series B'!$C11+'Series B'!$C12+'Series B'!$L12+'Series B'!$Q12)</f>
+        <v>139256350.0235261</v>
+      </c>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A65" s="1"/>
+      <c r="B65" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C65" s="1"/>
+      <c r="D65" s="1"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="1"/>
+      <c r="H65" s="1"/>
+      <c r="I65" s="88">
+        <f ca="1">I$47*'Series B'!$E15+I$48*'Series B'!$J15+I$49*'Series B'!$O15+I$50*'Series B'!$C15</f>
+        <v>24641255.718132924</v>
+      </c>
+      <c r="J65" s="88">
+        <f ca="1">J$47*'Series B'!$E15+J$48*'Series B'!$J15+J$49*'Series B'!$O15+J$50*'Series B'!$C15</f>
+        <v>32369750.028990984</v>
+      </c>
+      <c r="K65" s="88">
+        <f ca="1">K$47*'Series B'!$E15+K$48*'Series B'!$J15+K$49*'Series B'!$O15+K$50*'Series B'!$C15</f>
+        <v>40462187.53623873</v>
+      </c>
+      <c r="L65" s="88">
+        <f ca="1">L$47*'Series B'!$E15+L$48*'Series B'!$J15+L$49*'Series B'!$O15+L$50*'Series B'!$C15</f>
+        <v>48554625.043486476</v>
+      </c>
+      <c r="M65" s="88">
+        <f ca="1">M$47*'Series B'!$E15+M$48*'Series B'!$J15+M$49*'Series B'!$O15+M$50*'Series B'!$C15</f>
+        <v>56647062.550734229</v>
+      </c>
+      <c r="N65" s="88">
+        <f ca="1">N$47*'Series B'!$E15+N$48*'Series B'!$J15+N$49*'Series B'!$O15+N$50*'Series B'!$C15</f>
+        <v>64739500.057981968</v>
+      </c>
+      <c r="O65" s="88">
+        <f ca="1">O$47*'Series B'!$E15+O$48*'Series B'!$J15+O$49*'Series B'!$O15+O$50*'Series B'!$C15</f>
+        <v>80924375.07247746</v>
+      </c>
+      <c r="P65" s="88">
+        <f ca="1">P$47*'Series B'!$E15+P$48*'Series B'!$J15+P$49*'Series B'!$O15+P$50*'Series B'!$C15</f>
+        <v>121386562.60871619</v>
+      </c>
+    </row>
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A66" s="1"/>
+      <c r="B66" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C66" s="1"/>
+      <c r="D66" s="1"/>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1"/>
+      <c r="G66" s="1"/>
+      <c r="H66" s="1"/>
+      <c r="I66" s="88">
+        <f ca="1">I$47*'Series B'!$E16+I$48*'Series B'!$J16+I$49*'Series B'!$O16+I$50*'Series B'!$C16</f>
+        <v>3518298.6828376139</v>
+      </c>
+      <c r="J66" s="88">
+        <f ca="1">J$47*'Series B'!$E16+J$48*'Series B'!$J16+J$49*'Series B'!$O16+J$50*'Series B'!$C16</f>
+        <v>4621778.5954602547</v>
+      </c>
+      <c r="K66" s="88">
+        <f ca="1">K$47*'Series B'!$E16+K$48*'Series B'!$J16+K$49*'Series B'!$O16+K$50*'Series B'!$C16</f>
+        <v>5777223.2443253184</v>
+      </c>
+      <c r="L66" s="88">
+        <f ca="1">L$47*'Series B'!$E16+L$48*'Series B'!$J16+L$49*'Series B'!$O16+L$50*'Series B'!$C16</f>
+        <v>6932667.893190382</v>
+      </c>
+      <c r="M66" s="88">
+        <f ca="1">M$47*'Series B'!$E16+M$48*'Series B'!$J16+M$49*'Series B'!$O16+M$50*'Series B'!$C16</f>
+        <v>8088112.5420554457</v>
+      </c>
+      <c r="N66" s="88">
+        <f ca="1">N$47*'Series B'!$E16+N$48*'Series B'!$J16+N$49*'Series B'!$O16+N$50*'Series B'!$C16</f>
+        <v>9243557.1909205094</v>
+      </c>
+      <c r="O66" s="88">
+        <f ca="1">O$47*'Series B'!$E16+O$48*'Series B'!$J16+O$49*'Series B'!$O16+O$50*'Series B'!$C16</f>
+        <v>11554446.488650637</v>
+      </c>
+      <c r="P66" s="88">
+        <f ca="1">P$47*'Series B'!$E16+P$48*'Series B'!$J16+P$49*'Series B'!$O16+P$50*'Series B'!$C16</f>
+        <v>17331669.732975956</v>
+      </c>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A67" s="1"/>
+      <c r="B67" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C67" s="1"/>
+      <c r="D67" s="1"/>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1"/>
+      <c r="G67" s="1"/>
+      <c r="H67" s="1"/>
+      <c r="I67" s="88">
+        <f ca="1">I$47*'Series B'!$E17+I$48*'Series B'!$J17+I$49*'Series B'!$O17+I$50*'Series B'!$C17</f>
+        <v>22124641.051647268</v>
+      </c>
+      <c r="J67" s="88">
+        <f ca="1">J$47*'Series B'!$E17+J$48*'Series B'!$J17+J$49*'Series B'!$O17+J$50*'Series B'!$C17</f>
+        <v>29063822.839694299</v>
+      </c>
+      <c r="K67" s="88">
+        <f ca="1">K$47*'Series B'!$E17+K$48*'Series B'!$J17+K$49*'Series B'!$O17+K$50*'Series B'!$C17</f>
+        <v>36329778.549617872</v>
+      </c>
+      <c r="L67" s="88">
+        <f ca="1">L$47*'Series B'!$E17+L$48*'Series B'!$J17+L$49*'Series B'!$O17+L$50*'Series B'!$C17</f>
+        <v>43595734.259541452</v>
+      </c>
+      <c r="M67" s="88">
+        <f ca="1">M$47*'Series B'!$E17+M$48*'Series B'!$J17+M$49*'Series B'!$O17+M$50*'Series B'!$C17</f>
+        <v>50861689.969465025</v>
+      </c>
+      <c r="N67" s="88">
+        <f ca="1">N$47*'Series B'!$E17+N$48*'Series B'!$J17+N$49*'Series B'!$O17+N$50*'Series B'!$C17</f>
+        <v>58127645.679388598</v>
+      </c>
+      <c r="O67" s="88">
+        <f ca="1">O$47*'Series B'!$E17+O$48*'Series B'!$J17+O$49*'Series B'!$O17+O$50*'Series B'!$C17</f>
+        <v>72659557.099235743</v>
+      </c>
+      <c r="P67" s="88">
+        <f ca="1">P$47*'Series B'!$E17+P$48*'Series B'!$J17+P$49*'Series B'!$O17+P$50*'Series B'!$C17</f>
+        <v>108989335.64885363</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A68" s="1"/>
+      <c r="B68" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="I68" s="88">
+        <f ca="1">I$47*'Series B'!$E18+I$48*'Series B'!$J18+I$49*'Series B'!$O18+I$50*'Series B'!$C18</f>
+        <v>5531161.7165764151</v>
+      </c>
+      <c r="J68" s="88">
+        <f ca="1">J$47*'Series B'!$E18+J$48*'Series B'!$J18+J$49*'Series B'!$O18+J$50*'Series B'!$C18</f>
+        <v>7265957.7366176676</v>
+      </c>
+      <c r="K68" s="88">
+        <f ca="1">K$47*'Series B'!$E18+K$48*'Series B'!$J18+K$49*'Series B'!$O18+K$50*'Series B'!$C18</f>
+        <v>9082447.1707720831</v>
+      </c>
+      <c r="L68" s="88">
+        <f ca="1">L$47*'Series B'!$E18+L$48*'Series B'!$J18+L$49*'Series B'!$O18+L$50*'Series B'!$C18</f>
+        <v>10898936.6049265</v>
+      </c>
+      <c r="M68" s="88">
+        <f ca="1">M$47*'Series B'!$E18+M$48*'Series B'!$J18+M$49*'Series B'!$O18+M$50*'Series B'!$C18</f>
+        <v>12715426.039080918</v>
+      </c>
+      <c r="N68" s="88">
+        <f ca="1">N$47*'Series B'!$E18+N$48*'Series B'!$J18+N$49*'Series B'!$O18+N$50*'Series B'!$C18</f>
+        <v>14531915.473235335</v>
+      </c>
+      <c r="O68" s="88">
+        <f ca="1">O$47*'Series B'!$E18+O$48*'Series B'!$J18+O$49*'Series B'!$O18+O$50*'Series B'!$C18</f>
+        <v>18164894.341544166</v>
+      </c>
+      <c r="P68" s="88">
+        <f ca="1">P$47*'Series B'!$E18+P$48*'Series B'!$J18+P$49*'Series B'!$O18+P$50*'Series B'!$C18</f>
+        <v>27247341.512316253</v>
+      </c>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A69" s="1"/>
+      <c r="B69" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C69" s="1"/>
+      <c r="D69" s="1"/>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1"/>
+      <c r="G69" s="1"/>
+      <c r="H69" s="1"/>
+      <c r="I69" s="88">
+        <f ca="1">I$47*'Series B'!$E19+I$48*'Series B'!$J19+I$49*'Series B'!$O19+I$50*'Series B'!$C19</f>
+        <v>15000002.210399998</v>
+      </c>
+      <c r="J69" s="88">
+        <f ca="1">J$47*'Series B'!$E19+J$48*'Series B'!$J19+J$49*'Series B'!$O19+J$50*'Series B'!$C19</f>
+        <v>16416684.231348798</v>
+      </c>
+      <c r="K69" s="88">
+        <f ca="1">K$47*'Series B'!$E19+K$48*'Series B'!$J19+K$49*'Series B'!$O19+K$50*'Series B'!$C19</f>
+        <v>20520855.289185997</v>
+      </c>
+      <c r="L69" s="88">
+        <f ca="1">L$47*'Series B'!$E19+L$48*'Series B'!$J19+L$49*'Series B'!$O19+L$50*'Series B'!$C19</f>
+        <v>24625026.347023197</v>
+      </c>
+      <c r="M69" s="88">
+        <f ca="1">M$47*'Series B'!$E19+M$48*'Series B'!$J19+M$49*'Series B'!$O19+M$50*'Series B'!$C19</f>
+        <v>28729197.404860396</v>
+      </c>
+      <c r="N69" s="88">
+        <f ca="1">N$47*'Series B'!$E19+N$48*'Series B'!$J19+N$49*'Series B'!$O19+N$50*'Series B'!$C19</f>
+        <v>32833368.462697595</v>
+      </c>
+      <c r="O69" s="88">
+        <f ca="1">O$47*'Series B'!$E19+O$48*'Series B'!$J19+O$49*'Series B'!$O19+O$50*'Series B'!$C19</f>
+        <v>41041710.578371994</v>
+      </c>
+      <c r="P69" s="88">
+        <f ca="1">P$47*'Series B'!$E19+P$48*'Series B'!$J19+P$49*'Series B'!$O19+P$50*'Series B'!$C19</f>
+        <v>61562565.867557988</v>
+      </c>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A70" s="1"/>
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1"/>
+      <c r="G70" s="1"/>
+      <c r="H70" s="1"/>
+      <c r="I70" s="88"/>
+      <c r="J70" s="88"/>
+      <c r="K70" s="88"/>
+      <c r="L70" s="88"/>
+      <c r="M70" s="88"/>
+      <c r="N70" s="88"/>
+      <c r="O70" s="88"/>
+      <c r="P70" s="88"/>
+    </row>
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A71" s="1"/>
+      <c r="B71" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C71" s="1"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="88">
+        <f ca="1">SUM(I61:I69)-I16</f>
+        <v>0</v>
+      </c>
+      <c r="J71" s="88">
+        <f ca="1">SUM(J61:J69)-J16</f>
+        <v>0</v>
+      </c>
+      <c r="K71" s="88">
+        <f ca="1">SUM(K61:K69)-K16</f>
+        <v>0</v>
+      </c>
+      <c r="L71" s="88">
+        <f ca="1">SUM(L61:L69)-L16</f>
+        <v>0</v>
+      </c>
+      <c r="M71" s="88">
+        <f ca="1">SUM(M61:M69)-M16</f>
+        <v>0</v>
+      </c>
+      <c r="N71" s="88">
+        <f ca="1">SUM(N61:N69)-N16</f>
+        <v>0</v>
+      </c>
+      <c r="O71" s="88">
+        <f ca="1">SUM(O61:O69)-O16</f>
+        <v>0</v>
+      </c>
+      <c r="P71" s="88">
+        <f ca="1">SUM(P61:P69)-P16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A72" s="1"/>
+      <c r="B72" s="1"/>
+      <c r="C72" s="1"/>
+      <c r="D72" s="1"/>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1"/>
+      <c r="G72" s="1"/>
+      <c r="H72" s="1"/>
+      <c r="I72" s="56"/>
+      <c r="J72" s="56"/>
+      <c r="K72" s="56"/>
+      <c r="L72" s="56"/>
+      <c r="M72" s="56"/>
+      <c r="N72" s="56"/>
+      <c r="O72" s="56"/>
+      <c r="P72" s="56"/>
+    </row>
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A73" s="1"/>
+      <c r="B73" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C73" s="95"/>
+      <c r="D73" s="95"/>
+      <c r="E73" s="95"/>
+      <c r="F73" s="95"/>
+      <c r="G73" s="95"/>
+      <c r="H73" s="95"/>
+      <c r="I73" s="96"/>
+      <c r="J73" s="96"/>
+      <c r="K73" s="96"/>
+      <c r="L73" s="96"/>
+      <c r="M73" s="96"/>
+      <c r="N73" s="96"/>
+      <c r="O73" s="96"/>
+      <c r="P73" s="96"/>
+    </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A74" s="1"/>
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1"/>
+      <c r="G74" s="1"/>
+      <c r="H74" s="1"/>
+      <c r="I74" s="56"/>
+      <c r="J74" s="56"/>
+      <c r="K74" s="56"/>
+      <c r="L74" s="56"/>
+      <c r="M74" s="56"/>
+      <c r="N74" s="56"/>
+      <c r="O74" s="56"/>
+      <c r="P74" s="56"/>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A75" s="1"/>
+      <c r="B75" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
+      <c r="I75" s="88">
+        <f ca="1">I67</f>
+        <v>22124641.051647268</v>
+      </c>
+      <c r="J75" s="88">
+        <f ca="1">J67</f>
+        <v>29063822.839694299</v>
+      </c>
+      <c r="K75" s="88">
+        <f ca="1">K67</f>
+        <v>36329778.549617872</v>
+      </c>
+      <c r="L75" s="88">
+        <f ca="1">L67</f>
+        <v>43595734.259541452</v>
+      </c>
+      <c r="M75" s="88">
+        <f ca="1">M67</f>
+        <v>50861689.969465025</v>
+      </c>
+      <c r="N75" s="88">
+        <f ca="1">N67</f>
+        <v>58127645.679388598</v>
+      </c>
+      <c r="O75" s="88">
+        <f ca="1">O67</f>
+        <v>72659557.099235743</v>
+      </c>
+      <c r="P75" s="88">
+        <f ca="1">P67</f>
+        <v>108989335.64885363</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A76" s="1"/>
+      <c r="B76" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
+      <c r="I76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="J76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="K76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="L76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="M76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="N76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="O76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+      <c r="P76" s="97">
+        <f ca="1">'Series A'!$I$17+'Series B'!$N$17</f>
+        <v>17945847.858574606</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A77" s="1"/>
+      <c r="B77" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+      <c r="H77" s="1"/>
+      <c r="I77" s="88">
+        <f ca="1">I75-I76</f>
+        <v>4178793.1930726618</v>
+      </c>
+      <c r="J77" s="88">
+        <f ca="1">J75-J76</f>
+        <v>11117974.981119692</v>
+      </c>
+      <c r="K77" s="88">
+        <f ca="1">K75-K76</f>
+        <v>18383930.691043265</v>
+      </c>
+      <c r="L77" s="88">
+        <f ca="1">L75-L76</f>
+        <v>25649886.400966845</v>
+      </c>
+      <c r="M77" s="88">
+        <f ca="1">M75-M76</f>
+        <v>32915842.110890418</v>
+      </c>
+      <c r="N77" s="88">
+        <f ca="1">N75-N76</f>
+        <v>40181797.820813991</v>
+      </c>
+      <c r="O77" s="88">
+        <f ca="1">O75-O76</f>
+        <v>54713709.240661137</v>
+      </c>
+      <c r="P77" s="88">
+        <f ca="1">P75-P76</f>
+        <v>91043487.790279031</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A78" s="1"/>
+      <c r="B78" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C78" s="1"/>
+      <c r="D78" s="1"/>
+      <c r="E78" s="1"/>
+      <c r="F78" s="1"/>
+      <c r="G78" s="1"/>
+      <c r="H78" s="1"/>
+      <c r="I78" s="92">
+        <f ca="1">I75/I76</f>
+        <v>1.2328557126976876</v>
+      </c>
+      <c r="J78" s="92">
+        <f ca="1">J75/J76</f>
+        <v>1.6195291004769927</v>
+      </c>
+      <c r="K78" s="92">
+        <f ca="1">K75/K76</f>
+        <v>2.024411375596241</v>
+      </c>
+      <c r="L78" s="92">
+        <f ca="1">L75/L76</f>
+        <v>2.4292936507154894</v>
+      </c>
+      <c r="M78" s="92">
+        <f ca="1">M75/M76</f>
+        <v>2.8341759258347374</v>
+      </c>
+      <c r="N78" s="92">
+        <f ca="1">N75/N76</f>
+        <v>3.2390582009539854</v>
+      </c>
+      <c r="O78" s="92">
+        <f ca="1">O75/O76</f>
+        <v>4.0488227511924819</v>
+      </c>
+      <c r="P78" s="92">
+        <f ca="1">P75/P76</f>
+        <v>6.0732341267887229</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A79" s="1"/>
+      <c r="B79" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C79" s="1"/>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1"/>
+      <c r="G79" s="1"/>
+      <c r="H79" s="1"/>
+      <c r="I79" s="92">
+        <f ca="1">I48/'Series A'!$J$22</f>
+        <v>1.3482327931673459</v>
+      </c>
+      <c r="J79" s="92">
+        <f ca="1">J48/'Series A'!$J$22</f>
+        <v>1.8797014394241687</v>
+      </c>
+      <c r="K79" s="92">
+        <f ca="1">K48/'Series A'!$J$22</f>
+        <v>2.3496267992802107</v>
+      </c>
+      <c r="L79" s="92">
+        <f ca="1">L48/'Series A'!$J$22</f>
+        <v>2.8195521591362529</v>
+      </c>
+      <c r="M79" s="92">
+        <f ca="1">M48/'Series A'!$J$22</f>
+        <v>3.2894775189922951</v>
+      </c>
+      <c r="N79" s="92">
+        <f ca="1">N48/'Series A'!$J$22</f>
+        <v>3.7594028788483373</v>
+      </c>
+      <c r="O79" s="92">
+        <f ca="1">O48/'Series A'!$J$22</f>
+        <v>4.6992535985604214</v>
+      </c>
+      <c r="P79" s="92">
+        <f ca="1">P48/'Series A'!$J$22</f>
+        <v>7.0488803978406329</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A80" s="1"/>
+      <c r="B80" s="1"/>
+      <c r="C80" s="1"/>
+      <c r="D80" s="1"/>
+      <c r="E80" s="1"/>
+      <c r="F80" s="1"/>
+      <c r="G80" s="1"/>
+      <c r="H80" s="1"/>
+      <c r="I80" s="56"/>
+      <c r="J80" s="56"/>
+      <c r="K80" s="56"/>
+      <c r="L80" s="56"/>
+      <c r="M80" s="56"/>
+      <c r="N80" s="56"/>
+      <c r="O80" s="56"/>
+      <c r="P80" s="56"/>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A81" s="1"/>
+      <c r="B81" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C81" s="1"/>
+      <c r="D81" s="1"/>
+      <c r="E81" s="1"/>
+      <c r="F81" s="1"/>
+      <c r="G81" s="1"/>
+      <c r="H81" s="1"/>
+      <c r="I81" s="93">
+        <f ca="1">XIRR(I83:I85,$D$83:$D$85)</f>
+        <v>5.8570984005928042E-2</v>
+      </c>
+      <c r="J81" s="93">
+        <f ca="1">XIRR(J83:J85,$D$83:$D$85)</f>
+        <v>0.13975443243980409</v>
+      </c>
+      <c r="K81" s="93">
+        <f ca="1">XIRR(K83:K85,$D$83:$D$85)</f>
+        <v>0.21048800349235539</v>
+      </c>
+      <c r="L81" s="93">
+        <f ca="1">XIRR(L83:L85,$D$83:$D$85)</f>
+        <v>0.27133831381797791</v>
+      </c>
+      <c r="M81" s="93">
+        <f ca="1">XIRR(M83:M85,$D$83:$D$85)</f>
+        <v>0.32503222823143008</v>
+      </c>
+      <c r="N81" s="93">
+        <f ca="1">XIRR(N83:N85,$D$83:$D$85)</f>
+        <v>0.37327285408973698</v>
+      </c>
+      <c r="O81" s="93">
+        <f ca="1">XIRR(O83:O85,$D$83:$D$85)</f>
+        <v>0.45762366652488717</v>
+      </c>
+      <c r="P81" s="93">
+        <f ca="1">XIRR(P83:P85,$D$83:$D$85)</f>
+        <v>0.62363980412483222</v>
+      </c>
+    </row>
+    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A82" s="1"/>
+      <c r="B82" s="1"/>
+      <c r="C82" s="1"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="1"/>
+      <c r="F82" s="1"/>
+      <c r="G82" s="1"/>
+      <c r="H82" s="1"/>
+      <c r="I82" s="56"/>
+      <c r="J82" s="56"/>
+      <c r="K82" s="56"/>
+      <c r="L82" s="56"/>
+      <c r="M82" s="56"/>
+      <c r="N82" s="56"/>
+      <c r="O82" s="56"/>
+      <c r="P82" s="56"/>
+    </row>
+    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A83" s="1"/>
+      <c r="B83" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D83" s="84">
+        <v>46113</v>
+      </c>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1"/>
+      <c r="G83" s="1"/>
+      <c r="H83" s="1"/>
+      <c r="I83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="J83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="K83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="L83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="M83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="N83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="O83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+      <c r="P83" s="88">
+        <f>-'Series A'!$I$17</f>
+        <v>-12000000</v>
+      </c>
+    </row>
+    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A84" s="1"/>
+      <c r="B84" s="1"/>
+      <c r="C84" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D84" s="52">
+        <v>46478</v>
+      </c>
+      <c r="E84" s="1"/>
+      <c r="F84" s="1"/>
+      <c r="G84" s="1"/>
+      <c r="H84" s="1"/>
+      <c r="I84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="J84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="K84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="L84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="M84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="N84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="O84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+      <c r="P84" s="88">
+        <f ca="1">-'Series B'!$N$17</f>
+        <v>-5945847.8585746055</v>
+      </c>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A85" s="1"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D85" s="52">
+        <f>DATE(YEAR(D84)+3,MONTH(D84),DAY(D84))</f>
+        <v>47574</v>
+      </c>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1"/>
+      <c r="G85" s="1"/>
+      <c r="H85" s="1"/>
+      <c r="I85" s="88">
+        <f ca="1">I75</f>
+        <v>22124641.051647268</v>
+      </c>
+      <c r="J85" s="88">
+        <f ca="1">J75</f>
+        <v>29063822.839694299</v>
+      </c>
+      <c r="K85" s="88">
+        <f ca="1">K75</f>
+        <v>36329778.549617872</v>
+      </c>
+      <c r="L85" s="88">
+        <f ca="1">L75</f>
+        <v>43595734.259541452</v>
+      </c>
+      <c r="M85" s="88">
+        <f ca="1">M75</f>
+        <v>50861689.969465025</v>
+      </c>
+      <c r="N85" s="88">
+        <f ca="1">N75</f>
+        <v>58127645.679388598</v>
+      </c>
+      <c r="O85" s="88">
+        <f ca="1">O75</f>
+        <v>72659557.099235743</v>
+      </c>
+      <c r="P85" s="88">
+        <f ca="1">P75</f>
+        <v>108989335.64885363</v>
+      </c>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A86" s="1"/>
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1"/>
+      <c r="G86" s="1"/>
+      <c r="H86" s="1"/>
+      <c r="I86" s="1"/>
+      <c r="J86" s="1"/>
+      <c r="K86" s="1"/>
+      <c r="L86" s="1"/>
+      <c r="M86" s="1"/>
+      <c r="N86" s="1"/>
+      <c r="O86" s="1"/>
+      <c r="P86" s="1"/>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A87" s="1"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
+      <c r="G87" s="1"/>
+      <c r="H87" s="1"/>
+      <c r="I87" s="1"/>
+      <c r="J87" s="1"/>
+      <c r="K87" s="1"/>
+      <c r="L87" s="1"/>
+      <c r="M87" s="1"/>
+      <c r="N87" s="1"/>
+      <c r="O87" s="1"/>
+      <c r="P87" s="1"/>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A88" s="1"/>
+      <c r="B88" s="1"/>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1"/>
+      <c r="G88" s="1"/>
+      <c r="H88" s="1"/>
+      <c r="I88" s="1"/>
+      <c r="J88" s="1"/>
+      <c r="K88" s="1"/>
+      <c r="L88" s="1"/>
+      <c r="M88" s="1"/>
+      <c r="N88" s="1"/>
+      <c r="O88" s="1"/>
+      <c r="P88" s="1"/>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A89" s="1"/>
+      <c r="B89" s="1"/>
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1"/>
+      <c r="G89" s="1"/>
+      <c r="H89" s="1"/>
+      <c r="I89" s="1"/>
+      <c r="J89" s="1"/>
+      <c r="K89" s="1"/>
+      <c r="L89" s="1"/>
+      <c r="M89" s="1"/>
+      <c r="N89" s="1"/>
+      <c r="O89" s="1"/>
+      <c r="P89" s="1"/>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A90" s="1"/>
+      <c r="B90" s="1"/>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1"/>
+      <c r="G90" s="1"/>
+      <c r="H90" s="1"/>
+      <c r="I90" s="1"/>
+      <c r="J90" s="1"/>
+      <c r="K90" s="1"/>
+      <c r="L90" s="1"/>
+      <c r="M90" s="1"/>
+      <c r="N90" s="1"/>
+      <c r="O90" s="1"/>
+      <c r="P90" s="1"/>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A91" s="1"/>
+      <c r="B91" s="1"/>
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1"/>
+      <c r="G91" s="1"/>
+      <c r="H91" s="1"/>
+      <c r="I91" s="1"/>
+      <c r="J91" s="1"/>
+      <c r="K91" s="1"/>
+      <c r="L91" s="1"/>
+      <c r="M91" s="1"/>
+      <c r="N91" s="1"/>
+      <c r="O91" s="1"/>
+      <c r="P91" s="1"/>
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A92" s="1"/>
+      <c r="B92" s="1"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1"/>
+      <c r="G92" s="1"/>
+      <c r="H92" s="1"/>
+      <c r="I92" s="1"/>
+      <c r="J92" s="1"/>
+      <c r="K92" s="1"/>
+      <c r="L92" s="1"/>
+      <c r="M92" s="1"/>
+      <c r="N92" s="1"/>
+      <c r="O92" s="1"/>
+      <c r="P92" s="1"/>
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A93" s="1"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1"/>
+      <c r="G93" s="1"/>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1"/>
+      <c r="J93" s="1"/>
+      <c r="K93" s="1"/>
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+      <c r="N93" s="1"/>
+      <c r="O93" s="1"/>
+      <c r="P93" s="1"/>
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A94" s="1"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="1"/>
+      <c r="I94" s="1"/>
+      <c r="J94" s="1"/>
+      <c r="K94" s="1"/>
+      <c r="L94" s="1"/>
+      <c r="M94" s="1"/>
+      <c r="N94" s="1"/>
+      <c r="O94" s="1"/>
+      <c r="P94" s="1"/>
+    </row>
+    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A95" s="1"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1"/>
+      <c r="G95" s="1"/>
+      <c r="H95" s="1"/>
+      <c r="I95" s="1"/>
+      <c r="J95" s="1"/>
+      <c r="K95" s="1"/>
+      <c r="L95" s="1"/>
+      <c r="M95" s="1"/>
+      <c r="N95" s="1"/>
+      <c r="O95" s="1"/>
+      <c r="P95" s="1"/>
+    </row>
+    <row r="96" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A96" s="1"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1"/>
+      <c r="G96" s="1"/>
+      <c r="H96" s="1"/>
+      <c r="I96" s="1"/>
+      <c r="J96" s="1"/>
+      <c r="K96" s="1"/>
+      <c r="L96" s="1"/>
+      <c r="M96" s="1"/>
+      <c r="N96" s="1"/>
+      <c r="O96" s="1"/>
+      <c r="P96" s="1"/>
+    </row>
+    <row r="97" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A97" s="1"/>
+      <c r="B97" s="1"/>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+      <c r="E97" s="1"/>
+      <c r="F97" s="1"/>
+      <c r="G97" s="1"/>
+      <c r="H97" s="1"/>
+      <c r="I97" s="1"/>
+      <c r="J97" s="1"/>
+      <c r="K97" s="1"/>
+      <c r="L97" s="1"/>
+      <c r="M97" s="1"/>
+      <c r="N97" s="1"/>
+      <c r="O97" s="1"/>
+      <c r="P97" s="1"/>
+    </row>
+    <row r="98" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A98" s="1"/>
+      <c r="B98" s="1"/>
+      <c r="C98" s="1"/>
+      <c r="D98" s="1"/>
+      <c r="E98" s="1"/>
+      <c r="F98" s="1"/>
+      <c r="G98" s="1"/>
+      <c r="H98" s="1"/>
+      <c r="I98" s="1"/>
+      <c r="J98" s="1"/>
+      <c r="K98" s="1"/>
+      <c r="L98" s="1"/>
+      <c r="M98" s="1"/>
+      <c r="N98" s="1"/>
+      <c r="O98" s="1"/>
+      <c r="P98" s="1"/>
+    </row>
+    <row r="99" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A99" s="1"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+      <c r="H99" s="1"/>
+      <c r="I99" s="1"/>
+      <c r="J99" s="1"/>
+      <c r="K99" s="1"/>
+      <c r="L99" s="1"/>
+      <c r="M99" s="1"/>
+      <c r="N99" s="1"/>
+      <c r="O99" s="1"/>
+      <c r="P99" s="1"/>
+    </row>
+    <row r="100" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A100" s="1"/>
+      <c r="B100" s="1"/>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="1"/>
+      <c r="G100" s="1"/>
+      <c r="H100" s="1"/>
+      <c r="I100" s="1"/>
+      <c r="J100" s="1"/>
+      <c r="K100" s="1"/>
+      <c r="L100" s="1"/>
+      <c r="M100" s="1"/>
+      <c r="N100" s="1"/>
+      <c r="O100" s="1"/>
+      <c r="P100" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>